<commit_message>
Batch 3: purani character images sahi look ke hisaab se lagayi + character bank
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RVfDRs8Z25TZnX8xvhD7fv
</commit_message>
<xml_diff>
--- a/youtube stories/batch 3/Batch 3 - Production Sheet.xlsx
+++ b/youtube stories/batch 3/Batch 3 - Production Sheet.xlsx
@@ -812,7 +812,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Image Prompts sheet: HARA = purani image (nayi mat banao) – 72 alag images reuse. Baaki 68 nayi banani hain (BG_ wale long video 16:9 ke liye).</t>
+          <t>Image Prompts sheet: HARA = purani image (nayi mat banao) – 96 alag images reuse. Baaki 53 nayi banani hain (BG_ wale long video 16:9 ke liye).</t>
         </is>
       </c>
     </row>
@@ -3384,7 +3384,7 @@
       <c r="I11" s="16" t="inlineStr"/>
       <c r="J11" s="16" t="inlineStr">
         <is>
-          <t>A021_V_KAMLESH</t>
+          <t>C08-004_MR_RATHI</t>
         </is>
       </c>
       <c r="K11" s="16" t="inlineStr"/>
@@ -3449,7 +3449,7 @@
       </c>
       <c r="J12" s="16" t="inlineStr">
         <is>
-          <t>A021_V_KAMLESH</t>
+          <t>C08-004_MR_RATHI</t>
         </is>
       </c>
       <c r="K12" s="16" t="inlineStr"/>
@@ -3567,7 +3567,7 @@
       <c r="I14" s="16" t="inlineStr"/>
       <c r="J14" s="16" t="inlineStr">
         <is>
-          <t>P_KAANCH_TUKDE_CUT</t>
+          <t>P_KAANCH_TUKDE</t>
         </is>
       </c>
       <c r="K14" s="16" t="inlineStr">
@@ -4155,7 +4155,7 @@
       </c>
       <c r="J23" s="16" t="inlineStr">
         <is>
-          <t>G_W_MAROON_SAREE_CUT</t>
+          <t>C004_MAA</t>
         </is>
       </c>
       <c r="K23" s="16" t="inlineStr"/>
@@ -4221,7 +4221,7 @@
       </c>
       <c r="J24" s="17" t="inlineStr">
         <is>
-          <t>G_M_CAMERA_CUT</t>
+          <t>G_M_YELLOW_KURTA_CUT</t>
         </is>
       </c>
       <c r="K24" s="17" t="inlineStr"/>
@@ -4292,7 +4292,7 @@
       </c>
       <c r="J25" s="16" t="inlineStr">
         <is>
-          <t>G_V_MAN_GREY_CUT</t>
+          <t>C005_VICKY_KEY_CUT</t>
         </is>
       </c>
       <c r="K25" s="16" t="inlineStr"/>
@@ -4359,7 +4359,7 @@
       </c>
       <c r="J26" s="16" t="inlineStr">
         <is>
-          <t>C08-004_MR_RATHI</t>
+          <t>G_TTE</t>
         </is>
       </c>
       <c r="K26" s="16" t="inlineStr"/>
@@ -4425,7 +4425,7 @@
       </c>
       <c r="J27" s="16" t="inlineStr">
         <is>
-          <t>C004_SNEHA</t>
+          <t>C004_BEHEN</t>
         </is>
       </c>
       <c r="K27" s="16" t="inlineStr"/>
@@ -4877,7 +4877,7 @@
       <c r="I34" s="16" t="inlineStr"/>
       <c r="J34" s="16" t="inlineStr">
         <is>
-          <t>A022_V_RAO</t>
+          <t>C002_ARYAN</t>
         </is>
       </c>
       <c r="K34" s="16" t="inlineStr"/>
@@ -4942,7 +4942,7 @@
       </c>
       <c r="J35" s="16" t="inlineStr">
         <is>
-          <t>A022_V_RAO</t>
+          <t>C002_ARYAN</t>
         </is>
       </c>
       <c r="K35" s="16" t="inlineStr"/>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="J43" s="16" t="inlineStr">
         <is>
-          <t>C08-007_KAPOOR</t>
+          <t>G_M_OLD_NOGLASSES_CUT</t>
         </is>
       </c>
       <c r="K43" s="16" t="inlineStr"/>
@@ -5514,7 +5514,7 @@
       </c>
       <c r="J44" s="16" t="inlineStr">
         <is>
-          <t>C007_KAVYA</t>
+          <t>G_W_PINK_SUIT_CUT</t>
         </is>
       </c>
       <c r="K44" s="16" t="inlineStr"/>
@@ -5580,7 +5580,7 @@
       </c>
       <c r="J45" s="17" t="inlineStr">
         <is>
-          <t>G_V_MAN_CHECK_CUT</t>
+          <t>C007_VIKRAM</t>
         </is>
       </c>
       <c r="K45" s="17" t="inlineStr"/>
@@ -5651,7 +5651,7 @@
       </c>
       <c r="J46" s="16" t="inlineStr">
         <is>
-          <t>G_M_APRON_CUT</t>
+          <t>C017_CHEF</t>
         </is>
       </c>
       <c r="K46" s="16" t="inlineStr"/>
@@ -5718,7 +5718,7 @@
       </c>
       <c r="J47" s="16" t="inlineStr">
         <is>
-          <t>G_V_WOMAN_SAREE_CUT</t>
+          <t>C010_SUNITA</t>
         </is>
       </c>
       <c r="K47" s="16" t="inlineStr"/>
@@ -5785,7 +5785,7 @@
       </c>
       <c r="J48" s="16" t="inlineStr">
         <is>
-          <t>A022_JOHNNY</t>
+          <t>C015_MARCO</t>
         </is>
       </c>
       <c r="K48" s="16" t="inlineStr"/>
@@ -5851,7 +5851,7 @@
       </c>
       <c r="J49" s="16" t="inlineStr">
         <is>
-          <t>C04-010_ARJUN</t>
+          <t>G_M_LIGHTMAN_CUT</t>
         </is>
       </c>
       <c r="K49" s="16" t="inlineStr"/>
@@ -5984,7 +5984,7 @@
       </c>
       <c r="J51" s="16" t="inlineStr">
         <is>
-          <t>C005_NEHA</t>
+          <t>C018_SISTER</t>
         </is>
       </c>
       <c r="K51" s="16" t="inlineStr"/>
@@ -6045,7 +6045,7 @@
       <c r="I52" s="16" t="inlineStr"/>
       <c r="J52" s="16" t="inlineStr">
         <is>
-          <t>A022_JOHNNY</t>
+          <t>C015_MARCO</t>
         </is>
       </c>
       <c r="K52" s="16" t="inlineStr">
@@ -6436,7 +6436,7 @@
       <c r="I58" s="16" t="inlineStr"/>
       <c r="J58" s="16" t="inlineStr">
         <is>
-          <t>A023_V_DESHMUKH</t>
+          <t>G_V_MAN_GREY_CUT</t>
         </is>
       </c>
       <c r="K58" s="16" t="inlineStr"/>
@@ -6501,7 +6501,7 @@
       </c>
       <c r="J59" s="16" t="inlineStr">
         <is>
-          <t>A023_V_DESHMUKH</t>
+          <t>G_V_MAN_GREY_CUT</t>
         </is>
       </c>
       <c r="K59" s="16" t="inlineStr"/>
@@ -6863,7 +6863,7 @@
       <c r="I65" s="16" t="inlineStr"/>
       <c r="J65" s="16" t="inlineStr">
         <is>
-          <t>P_A023_BOTTLE</t>
+          <t>P_BOTTLE_CUT</t>
         </is>
       </c>
       <c r="K65" s="16" t="inlineStr">
@@ -7073,7 +7073,7 @@
       </c>
       <c r="J68" s="16" t="inlineStr">
         <is>
-          <t>A023_BALA</t>
+          <t>C18-003_PRATEEK</t>
         </is>
       </c>
       <c r="K68" s="16" t="inlineStr"/>
@@ -7272,7 +7272,7 @@
       </c>
       <c r="J71" s="16" t="inlineStr">
         <is>
-          <t>G_V_MAN_BLUE_CUT</t>
+          <t>C020_NOAH</t>
         </is>
       </c>
       <c r="K71" s="16" t="inlineStr"/>
@@ -7338,7 +7338,7 @@
       </c>
       <c r="J72" s="16" t="inlineStr">
         <is>
-          <t>A023_ROY</t>
+          <t>G_CIVIL_RED_CUT</t>
         </is>
       </c>
       <c r="K72" s="16" t="inlineStr"/>
@@ -7388,7 +7388,7 @@
       </c>
       <c r="G73" s="16" t="inlineStr">
         <is>
-          <t>क्रिकेटर सोहम। प्रेसिडेंट ने टीम से निकाला। बोले... मैं टी-ट्वेंटी मैच खेल रहा था। हर टीम को बीस ओवर।</t>
+          <t>क्रिकेटर मनोज। प्रेसिडेंट ने टीम से निकाला। बोले... मैं टी-ट्वेंटी मैच खेल रहा था। हर टीम को बीस ओवर।</t>
         </is>
       </c>
       <c r="H73" s="16" t="inlineStr">
@@ -7399,13 +7399,13 @@
       <c r="I73" s="16" t="inlineStr">
         <is>
           <t>SUSPECT 7/10
-Cricketer Soham
+Cricketer Manoj
 (team se nikala)</t>
         </is>
       </c>
       <c r="J73" s="16" t="inlineStr">
         <is>
-          <t>G_CR_VIKRAM_CUT</t>
+          <t>G_CR_MANOJ_CUT</t>
         </is>
       </c>
       <c r="K73" s="16" t="inlineStr"/>
@@ -7471,7 +7471,7 @@
       </c>
       <c r="J74" s="17" t="inlineStr">
         <is>
-          <t>A023_AJINKYA</t>
+          <t>G_CIVIL_GREEN_CUT</t>
         </is>
       </c>
       <c r="K74" s="17" t="inlineStr"/>
@@ -7541,7 +7541,7 @@
       </c>
       <c r="J75" s="16" t="inlineStr">
         <is>
-          <t>G_W_PINK_SUIT_CUT</t>
+          <t>A023_KAPOOR</t>
         </is>
       </c>
       <c r="K75" s="16" t="inlineStr"/>
@@ -7607,7 +7607,7 @@
       </c>
       <c r="J76" s="16" t="inlineStr">
         <is>
-          <t>C008_NEHA</t>
+          <t>A023_SAINA</t>
         </is>
       </c>
       <c r="K76" s="16" t="inlineStr"/>
@@ -8059,7 +8059,7 @@
       <c r="I83" s="16" t="inlineStr"/>
       <c r="J83" s="16" t="inlineStr">
         <is>
-          <t>A024_V_PANDEY</t>
+          <t>C04-008_GUPTA_SLUMPED</t>
         </is>
       </c>
       <c r="K83" s="16" t="inlineStr"/>
@@ -8124,7 +8124,7 @@
       </c>
       <c r="J84" s="16" t="inlineStr">
         <is>
-          <t>A024_V_PANDEY</t>
+          <t>C04-008_GUPTA_SLUMPED</t>
         </is>
       </c>
       <c r="K84" s="16" t="inlineStr"/>
@@ -8630,7 +8630,7 @@
       </c>
       <c r="J92" s="16" t="inlineStr">
         <is>
-          <t>C010_SUNITA</t>
+          <t>G_W_MAROON_SAREE_CUT</t>
         </is>
       </c>
       <c r="K92" s="16" t="inlineStr"/>
@@ -8763,7 +8763,7 @@
       </c>
       <c r="J94" s="16" t="inlineStr">
         <is>
-          <t>C004_BEHEN</t>
+          <t>C002_RIYA_CUT</t>
         </is>
       </c>
       <c r="K94" s="16" t="inlineStr"/>
@@ -8830,7 +8830,7 @@
       </c>
       <c r="J95" s="16" t="inlineStr">
         <is>
-          <t>C004_PADOSI</t>
+          <t>C12-010_MAHESH</t>
         </is>
       </c>
       <c r="K95" s="16" t="inlineStr"/>
@@ -8896,7 +8896,7 @@
       </c>
       <c r="J96" s="16" t="inlineStr">
         <is>
-          <t>G_V_MAN_BLUE_CUT</t>
+          <t>C003_SURAJ_CUT</t>
         </is>
       </c>
       <c r="K96" s="16" t="inlineStr"/>
@@ -8962,7 +8962,7 @@
       </c>
       <c r="J97" s="17" t="inlineStr">
         <is>
-          <t>G_M_YELLOW_KURTA_CUT</t>
+          <t>C001_ROHIT</t>
         </is>
       </c>
       <c r="K97" s="17" t="inlineStr"/>
@@ -9099,7 +9099,7 @@
       </c>
       <c r="J99" s="16" t="inlineStr">
         <is>
-          <t>G_M_LIGHTMAN_CUT</t>
+          <t>G_M_BLUE_SHIRT_CUT</t>
         </is>
       </c>
       <c r="K99" s="16" t="inlineStr"/>
@@ -9551,7 +9551,7 @@
       <c r="I106" s="16" t="inlineStr"/>
       <c r="J106" s="16" t="inlineStr">
         <is>
-          <t>A025_V_KHAN</t>
+          <t>G_V_MAN_CHECK_CUT</t>
         </is>
       </c>
       <c r="K106" s="16" t="inlineStr"/>
@@ -9616,7 +9616,7 @@
       </c>
       <c r="J107" s="16" t="inlineStr">
         <is>
-          <t>A025_V_KHAN</t>
+          <t>G_V_MAN_CHECK_CUT</t>
         </is>
       </c>
       <c r="K107" s="16" t="inlineStr"/>
@@ -10122,7 +10122,7 @@
       </c>
       <c r="J115" s="16" t="inlineStr">
         <is>
-          <t>C001_ROHIT</t>
+          <t>G_CR_ROHIT_CUT</t>
         </is>
       </c>
       <c r="K115" s="16" t="inlineStr"/>
@@ -10188,7 +10188,7 @@
       </c>
       <c r="J116" s="17" t="inlineStr">
         <is>
-          <t>G_M_BROWN_JACKET_CUT</t>
+          <t>G_M_CAMERA_CUT</t>
         </is>
       </c>
       <c r="K116" s="17" t="inlineStr"/>
@@ -10259,7 +10259,7 @@
       </c>
       <c r="J117" s="16" t="inlineStr">
         <is>
-          <t>C004_SNEHA</t>
+          <t>C002_POOJA</t>
         </is>
       </c>
       <c r="K117" s="16" t="inlineStr"/>
@@ -10309,7 +10309,7 @@
       </c>
       <c r="G118" s="16" t="inlineStr">
         <is>
-          <t>गाइड भूपेंद्र। बोले... मैं राजस्थान के रणथंभौर में था, बाघ के पीछे जीप दौड़ा रहा था।</t>
+          <t>गाइड कल्लू। बोले... मैं राजस्थान के रणथंभौर में था, बाघ के पीछे जीप दौड़ा रहा था।</t>
         </is>
       </c>
       <c r="H118" s="16" t="inlineStr">
@@ -10320,12 +10320,12 @@
       <c r="I118" s="16" t="inlineStr">
         <is>
           <t>SUSPECT 4/9
-Guide Bhupendra</t>
+Guide Kallu</t>
         </is>
       </c>
       <c r="J118" s="16" t="inlineStr">
         <is>
-          <t>A025_BHUPENDRA</t>
+          <t>G_KALLU_CUT</t>
         </is>
       </c>
       <c r="K118" s="16" t="inlineStr"/>
@@ -10391,7 +10391,7 @@
       </c>
       <c r="J119" s="16" t="inlineStr">
         <is>
-          <t>C001_ANJALI</t>
+          <t>C011_EMMA</t>
         </is>
       </c>
       <c r="K119" s="16" t="inlineStr"/>
@@ -10458,7 +10458,7 @@
       </c>
       <c r="J120" s="16" t="inlineStr">
         <is>
-          <t>G_V_MAN_SHERWANI_CUT</t>
+          <t>C013_LAWYER</t>
         </is>
       </c>
       <c r="K120" s="16" t="inlineStr"/>
@@ -10718,7 +10718,7 @@
       <c r="I124" s="16" t="inlineStr"/>
       <c r="J124" s="16" t="inlineStr">
         <is>
-          <t>C001_ROHIT</t>
+          <t>G_CR_ROHIT_CUT</t>
         </is>
       </c>
       <c r="K124" s="16" t="inlineStr">
@@ -11109,7 +11109,7 @@
       <c r="I130" s="16" t="inlineStr"/>
       <c r="J130" s="16" t="inlineStr">
         <is>
-          <t>A026_V_TSERING</t>
+          <t>C001_VIKAS</t>
         </is>
       </c>
       <c r="K130" s="16" t="inlineStr"/>
@@ -11174,7 +11174,7 @@
       </c>
       <c r="J131" s="16" t="inlineStr">
         <is>
-          <t>A026_V_TSERING</t>
+          <t>C001_VIKAS</t>
         </is>
       </c>
       <c r="K131" s="16" t="inlineStr"/>
@@ -11536,7 +11536,7 @@
       <c r="I137" s="16" t="inlineStr"/>
       <c r="J137" s="16" t="inlineStr">
         <is>
-          <t>P_A026_SHOES</t>
+          <t>P_SHOES</t>
         </is>
       </c>
       <c r="K137" s="16" t="inlineStr">
@@ -11730,7 +11730,7 @@
       </c>
       <c r="G140" s="16" t="inlineStr">
         <is>
-          <t>ब्लॉगर नेहा। बोलीं... मैं मेघालय के चेरापूंजी से आई, दुनिया की सबसे ज़्यादा बारिश वाली जगहों में से एक।</t>
+          <t>ब्लॉगर तन्वी। बोले... मैं मेघालय के चेरापूंजी से आई, दुनिया की सबसे ज़्यादा बारिश वाली जगहों में से एक।</t>
         </is>
       </c>
       <c r="H140" s="16" t="inlineStr">
@@ -11741,12 +11741,12 @@
       <c r="I140" s="16" t="inlineStr">
         <is>
           <t>SUSPECT 2/9
-Blogger Neha</t>
+Blogger Tanvi</t>
         </is>
       </c>
       <c r="J140" s="16" t="inlineStr">
         <is>
-          <t>C008_NEHA</t>
+          <t>G_TANVI</t>
         </is>
       </c>
       <c r="K140" s="16" t="inlineStr"/>
@@ -11812,7 +11812,7 @@
       </c>
       <c r="J141" s="16" t="inlineStr">
         <is>
-          <t>G_M_CAMERA_CUT</t>
+          <t>G_M_BROWN_JACKET_CUT</t>
         </is>
       </c>
       <c r="K141" s="16" t="inlineStr"/>
@@ -11879,7 +11879,7 @@
       </c>
       <c r="J142" s="16" t="inlineStr">
         <is>
-          <t>A026_KARMA</t>
+          <t>G_M_BLUE_JACKET_B_CUT</t>
         </is>
       </c>
       <c r="K142" s="16" t="inlineStr"/>
@@ -11945,7 +11945,7 @@
       </c>
       <c r="J143" s="16" t="inlineStr">
         <is>
-          <t>G_M_OLD_GLASSES_CUT</t>
+          <t>C006_GUPTA</t>
         </is>
       </c>
       <c r="K143" s="16" t="inlineStr"/>
@@ -12011,7 +12011,7 @@
       </c>
       <c r="J144" s="16" t="inlineStr">
         <is>
-          <t>C002_RIYA_CUT</t>
+          <t>C001_ANJALI</t>
         </is>
       </c>
       <c r="K144" s="16" t="inlineStr"/>
@@ -12078,7 +12078,7 @@
       </c>
       <c r="J145" s="16" t="inlineStr">
         <is>
-          <t>C16-001_DRMEHTA</t>
+          <t>G_M_OLD_GLASSES_CUT</t>
         </is>
       </c>
       <c r="K145" s="16" t="inlineStr"/>
@@ -12145,7 +12145,7 @@
       </c>
       <c r="J146" s="16" t="inlineStr">
         <is>
-          <t>A026_DORJEE</t>
+          <t>G_M_APRON_CUT</t>
         </is>
       </c>
       <c r="K146" s="16" t="inlineStr"/>
@@ -12211,7 +12211,7 @@
       </c>
       <c r="J147" s="17" t="inlineStr">
         <is>
-          <t>C007_VIKRAM</t>
+          <t>G_CIVIL_BLACK_CUT</t>
         </is>
       </c>
       <c r="K147" s="17" t="inlineStr"/>
@@ -12276,7 +12276,7 @@
       <c r="I148" s="16" t="inlineStr"/>
       <c r="J148" s="16" t="inlineStr">
         <is>
-          <t>A026_DORJEE</t>
+          <t>G_M_APRON_CUT</t>
         </is>
       </c>
       <c r="K148" s="16" t="inlineStr">
@@ -12667,7 +12667,7 @@
       <c r="I154" s="16" t="inlineStr"/>
       <c r="J154" s="16" t="inlineStr">
         <is>
-          <t>A027_V_MOHAPATRA</t>
+          <t>G_V_MAN_SHERWANI_CUT</t>
         </is>
       </c>
       <c r="K154" s="16" t="inlineStr"/>
@@ -12732,7 +12732,7 @@
       </c>
       <c r="J155" s="16" t="inlineStr">
         <is>
-          <t>A027_V_MOHAPATRA</t>
+          <t>G_V_MAN_SHERWANI_CUT</t>
         </is>
       </c>
       <c r="K155" s="16" t="inlineStr"/>
@@ -13238,7 +13238,7 @@
       </c>
       <c r="J163" s="16" t="inlineStr">
         <is>
-          <t>C002_POOJA</t>
+          <t>C019_COWORKER</t>
         </is>
       </c>
       <c r="K163" s="16" t="inlineStr"/>
@@ -13371,7 +13371,7 @@
       </c>
       <c r="J165" s="16" t="inlineStr">
         <is>
-          <t>C18-003_PRATEEK</t>
+          <t>C10-004_DEEPAK</t>
         </is>
       </c>
       <c r="K165" s="16" t="inlineStr"/>
@@ -13437,7 +13437,7 @@
       </c>
       <c r="J166" s="17" t="inlineStr">
         <is>
-          <t>C17-001_SETH</t>
+          <t>C017_BESTMAN</t>
         </is>
       </c>
       <c r="K166" s="17" t="inlineStr"/>
@@ -13508,7 +13508,7 @@
       </c>
       <c r="J167" s="16" t="inlineStr">
         <is>
-          <t>G_V_WOMAN_SAREE_CUT</t>
+          <t>C010_SUNITA</t>
         </is>
       </c>
       <c r="K167" s="16" t="inlineStr"/>
@@ -13574,7 +13574,7 @@
       </c>
       <c r="J168" s="16" t="inlineStr">
         <is>
-          <t>G_V_MAN_CHECK_CUT</t>
+          <t>C005_VICKY</t>
         </is>
       </c>
       <c r="K168" s="16" t="inlineStr"/>
@@ -13641,7 +13641,7 @@
       </c>
       <c r="J169" s="16" t="inlineStr">
         <is>
-          <t>C007_KAVYA</t>
+          <t>C004_BEHEN</t>
         </is>
       </c>
       <c r="K169" s="16" t="inlineStr"/>
@@ -13707,7 +13707,7 @@
       </c>
       <c r="J170" s="16" t="inlineStr">
         <is>
-          <t>G_V_MAN_GREY_CUT</t>
+          <t>C007_NIKHIL</t>
         </is>
       </c>
       <c r="K170" s="16" t="inlineStr"/>
@@ -13824,7 +13824,7 @@
       </c>
       <c r="G172" s="16" t="inlineStr">
         <is>
-          <t>सफ़ाईवाला रामू। बोले... मैं अमृतसर में जलियाँवाला बाग़ गया था।</t>
+          <t>सफ़ाईवाला गोपी। बोले... मैं अमृतसर में जलियाँवाला बाग़ गया था।</t>
         </is>
       </c>
       <c r="H172" s="16" t="inlineStr">
@@ -13835,12 +13835,12 @@
       <c r="I172" s="16" t="inlineStr">
         <is>
           <t>SUSPECT 10/10
-Safaiwala Ramu</t>
+Safaiwala Gopi</t>
         </is>
       </c>
       <c r="J172" s="16" t="inlineStr">
         <is>
-          <t>G_RAMU</t>
+          <t>G_M_GAMCHHA_CUT</t>
         </is>
       </c>
       <c r="K172" s="16" t="inlineStr"/>
@@ -14292,7 +14292,7 @@
       <c r="I179" s="16" t="inlineStr"/>
       <c r="J179" s="16" t="inlineStr">
         <is>
-          <t>A028_V_GREWAL</t>
+          <t>C08-007_KAPOOR</t>
         </is>
       </c>
       <c r="K179" s="16" t="inlineStr"/>
@@ -14357,7 +14357,7 @@
       </c>
       <c r="J180" s="16" t="inlineStr">
         <is>
-          <t>A028_V_GREWAL</t>
+          <t>C08-007_KAPOOR</t>
         </is>
       </c>
       <c r="K180" s="16" t="inlineStr"/>
@@ -14863,7 +14863,7 @@
       </c>
       <c r="J188" s="16" t="inlineStr">
         <is>
-          <t>C005_VICKY</t>
+          <t>C018_BOYFRIEND</t>
         </is>
       </c>
       <c r="K188" s="16" t="inlineStr"/>
@@ -15331,7 +15331,7 @@
       </c>
       <c r="J195" s="16" t="inlineStr">
         <is>
-          <t>C001_ANJALI</t>
+          <t>A028_ANU</t>
         </is>
       </c>
       <c r="K195" s="16" t="inlineStr"/>
@@ -15783,7 +15783,7 @@
       <c r="I202" s="16" t="inlineStr"/>
       <c r="J202" s="16" t="inlineStr">
         <is>
-          <t>C04-008_GUPTA_SLUMPED</t>
+          <t>C17-001_SETH</t>
         </is>
       </c>
       <c r="K202" s="16" t="inlineStr"/>
@@ -15848,7 +15848,7 @@
       </c>
       <c r="J203" s="16" t="inlineStr">
         <is>
-          <t>C04-008_GUPTA_SLUMPED</t>
+          <t>C17-001_SETH</t>
         </is>
       </c>
       <c r="K203" s="16" t="inlineStr"/>
@@ -16353,7 +16353,7 @@
       </c>
       <c r="J211" s="17" t="inlineStr">
         <is>
-          <t>C006_GUPTA</t>
+          <t>G_M_OLD_NOGLASSES_CUT</t>
         </is>
       </c>
       <c r="K211" s="17" t="inlineStr"/>
@@ -16424,7 +16424,7 @@
       </c>
       <c r="J212" s="16" t="inlineStr">
         <is>
-          <t>C004_AMIT</t>
+          <t>C003_BHATIJA</t>
         </is>
       </c>
       <c r="K212" s="16" t="inlineStr"/>
@@ -16490,7 +16490,7 @@
       </c>
       <c r="J213" s="16" t="inlineStr">
         <is>
-          <t>C004_SNEHA</t>
+          <t>C002_POOJA</t>
         </is>
       </c>
       <c r="K213" s="16" t="inlineStr"/>
@@ -16557,7 +16557,7 @@
       </c>
       <c r="J214" s="16" t="inlineStr">
         <is>
-          <t>C003_BHATIJA</t>
+          <t>C004_AMIT</t>
         </is>
       </c>
       <c r="K214" s="16" t="inlineStr"/>
@@ -16624,7 +16624,7 @@
       </c>
       <c r="J215" s="16" t="inlineStr">
         <is>
-          <t>G_V_MAN_BLUE_CUT</t>
+          <t>G_M_BLUE_JACKET_A_CUT</t>
         </is>
       </c>
       <c r="K215" s="16" t="inlineStr"/>
@@ -16757,7 +16757,7 @@
       </c>
       <c r="J217" s="16" t="inlineStr">
         <is>
-          <t>C08-004_MR_RATHI</t>
+          <t>C004_PADOSI</t>
         </is>
       </c>
       <c r="K217" s="16" t="inlineStr"/>
@@ -16950,7 +16950,7 @@
       <c r="I220" s="16" t="inlineStr"/>
       <c r="J220" s="16" t="inlineStr">
         <is>
-          <t>G_V_MAN_BLUE_CUT</t>
+          <t>G_M_BLUE_JACKET_A_CUT</t>
         </is>
       </c>
       <c r="K220" s="16" t="inlineStr">
@@ -17341,7 +17341,7 @@
       <c r="I226" s="16" t="inlineStr"/>
       <c r="J226" s="16" t="inlineStr">
         <is>
-          <t>A030_V_JOSHI</t>
+          <t>C04-010_ARJUN</t>
         </is>
       </c>
       <c r="K226" s="16" t="inlineStr"/>
@@ -17406,7 +17406,7 @@
       </c>
       <c r="J227" s="16" t="inlineStr">
         <is>
-          <t>A030_V_JOSHI</t>
+          <t>C04-010_ARJUN</t>
         </is>
       </c>
       <c r="K227" s="16" t="inlineStr"/>
@@ -17912,7 +17912,7 @@
       </c>
       <c r="J235" s="16" t="inlineStr">
         <is>
-          <t>G_M_GREY_HOODIE_CUT</t>
+          <t>C020_BROTHER</t>
         </is>
       </c>
       <c r="K235" s="16" t="inlineStr"/>
@@ -17978,7 +17978,7 @@
       </c>
       <c r="J236" s="16" t="inlineStr">
         <is>
-          <t>C005_NEHA</t>
+          <t>G_W_PINK_SUIT_CUT</t>
         </is>
       </c>
       <c r="K236" s="16" t="inlineStr"/>
@@ -18044,7 +18044,7 @@
       </c>
       <c r="J237" s="16" t="inlineStr">
         <is>
-          <t>G_M_OLD_NOGLASSES_CUT</t>
+          <t>C011_TOM</t>
         </is>
       </c>
       <c r="K237" s="16" t="inlineStr"/>
@@ -18111,7 +18111,7 @@
       </c>
       <c r="J238" s="16" t="inlineStr">
         <is>
-          <t>C007_KAVYA</t>
+          <t>C018_SISTER</t>
         </is>
       </c>
       <c r="K238" s="16" t="inlineStr"/>
@@ -18378,7 +18378,7 @@
       </c>
       <c r="J242" s="16" t="inlineStr">
         <is>
-          <t>C10-004_DEEPAK</t>
+          <t>C03-003_VICKY</t>
         </is>
       </c>
       <c r="K242" s="16" t="inlineStr"/>
@@ -18510,7 +18510,7 @@
       </c>
       <c r="J244" s="17" t="inlineStr">
         <is>
-          <t>G_V_MAN_CHECK_CUT</t>
+          <t>C008_GUEST</t>
         </is>
       </c>
       <c r="K244" s="17" t="inlineStr"/>
@@ -18575,7 +18575,7 @@
       <c r="I245" s="16" t="inlineStr"/>
       <c r="J245" s="16" t="inlineStr">
         <is>
-          <t>G_M_GREY_HOODIE_CUT</t>
+          <t>C020_BROTHER</t>
         </is>
       </c>
       <c r="K245" s="16" t="inlineStr">
@@ -20396,7 +20396,7 @@
       </c>
       <c r="H18" s="16" t="inlineStr">
         <is>
-          <t>A021_V_KAMLESH</t>
+          <t>C08-004_MR_RATHI</t>
         </is>
       </c>
       <c r="I18" s="16" t="inlineStr">
@@ -20469,7 +20469,7 @@
       </c>
       <c r="H19" s="16" t="inlineStr">
         <is>
-          <t>A021_V_KAMLESH</t>
+          <t>C08-004_MR_RATHI</t>
         </is>
       </c>
       <c r="I19" s="16" t="inlineStr">
@@ -20538,7 +20538,7 @@
       </c>
       <c r="H20" s="16" t="inlineStr">
         <is>
-          <t>A021_V_KAMLESH</t>
+          <t>C08-004_MR_RATHI</t>
         </is>
       </c>
       <c r="I20" s="16" t="inlineStr">
@@ -20615,7 +20615,7 @@
       </c>
       <c r="H21" s="16" t="inlineStr">
         <is>
-          <t>A021_V_KAMLESH</t>
+          <t>C08-004_MR_RATHI</t>
         </is>
       </c>
       <c r="I21" s="16" t="inlineStr">
@@ -20684,7 +20684,7 @@
       </c>
       <c r="H22" s="16" t="inlineStr">
         <is>
-          <t>A021_V_KAMLESH</t>
+          <t>C08-004_MR_RATHI</t>
         </is>
       </c>
       <c r="I22" s="16" t="inlineStr">
@@ -20822,7 +20822,7 @@
       <c r="G24" s="16" t="inlineStr"/>
       <c r="H24" s="16" t="inlineStr">
         <is>
-          <t>P_KAANCH_TUKDE_CUT</t>
+          <t>P_KAANCH_TUKDE</t>
         </is>
       </c>
       <c r="I24" s="16" t="inlineStr">
@@ -22031,7 +22031,7 @@
       </c>
       <c r="H40" s="16" t="inlineStr">
         <is>
-          <t>G_W_MAROON_SAREE_CUT</t>
+          <t>C004_MAA</t>
         </is>
       </c>
       <c r="I40" s="16" t="inlineStr">
@@ -22114,7 +22114,7 @@
       </c>
       <c r="H41" s="16" t="inlineStr">
         <is>
-          <t>G_W_MAROON_SAREE_CUT</t>
+          <t>C004_MAA</t>
         </is>
       </c>
       <c r="I41" s="16" t="inlineStr">
@@ -22187,7 +22187,7 @@
       </c>
       <c r="H42" s="16" t="inlineStr">
         <is>
-          <t>G_W_MAROON_SAREE_CUT</t>
+          <t>C004_MAA</t>
         </is>
       </c>
       <c r="I42" s="16" t="inlineStr">
@@ -22260,7 +22260,7 @@
       </c>
       <c r="H43" s="16" t="inlineStr">
         <is>
-          <t>G_M_CAMERA_CUT</t>
+          <t>G_M_YELLOW_KURTA_CUT</t>
         </is>
       </c>
       <c r="I43" s="16" t="inlineStr">
@@ -22342,7 +22342,7 @@
       </c>
       <c r="H44" s="16" t="inlineStr">
         <is>
-          <t>G_M_CAMERA_CUT</t>
+          <t>G_M_YELLOW_KURTA_CUT</t>
         </is>
       </c>
       <c r="I44" s="16" t="inlineStr">
@@ -22415,7 +22415,7 @@
       </c>
       <c r="H45" s="16" t="inlineStr">
         <is>
-          <t>G_M_CAMERA_CUT</t>
+          <t>G_M_YELLOW_KURTA_CUT</t>
         </is>
       </c>
       <c r="I45" s="16" t="inlineStr">
@@ -22488,7 +22488,7 @@
       </c>
       <c r="H46" s="16" t="inlineStr">
         <is>
-          <t>G_V_MAN_GREY_CUT</t>
+          <t>C005_VICKY_KEY_CUT</t>
         </is>
       </c>
       <c r="I46" s="16" t="inlineStr">
@@ -22571,7 +22571,7 @@
       </c>
       <c r="H47" s="16" t="inlineStr">
         <is>
-          <t>G_V_MAN_GREY_CUT</t>
+          <t>C005_VICKY_KEY_CUT</t>
         </is>
       </c>
       <c r="I47" s="16" t="inlineStr">
@@ -22644,7 +22644,7 @@
       </c>
       <c r="H48" s="16" t="inlineStr">
         <is>
-          <t>G_V_MAN_GREY_CUT</t>
+          <t>C005_VICKY_KEY_CUT</t>
         </is>
       </c>
       <c r="I48" s="16" t="inlineStr">
@@ -22717,7 +22717,7 @@
       </c>
       <c r="H49" s="16" t="inlineStr">
         <is>
-          <t>C08-004_MR_RATHI</t>
+          <t>G_TTE</t>
         </is>
       </c>
       <c r="I49" s="16" t="inlineStr">
@@ -22800,7 +22800,7 @@
       </c>
       <c r="H50" s="16" t="inlineStr">
         <is>
-          <t>C08-004_MR_RATHI</t>
+          <t>G_TTE</t>
         </is>
       </c>
       <c r="I50" s="16" t="inlineStr">
@@ -22873,7 +22873,7 @@
       </c>
       <c r="H51" s="16" t="inlineStr">
         <is>
-          <t>C08-004_MR_RATHI</t>
+          <t>G_TTE</t>
         </is>
       </c>
       <c r="I51" s="16" t="inlineStr">
@@ -22946,7 +22946,7 @@
       </c>
       <c r="H52" s="16" t="inlineStr">
         <is>
-          <t>C004_SNEHA</t>
+          <t>C004_BEHEN</t>
         </is>
       </c>
       <c r="I52" s="16" t="inlineStr">
@@ -23028,7 +23028,7 @@
       </c>
       <c r="H53" s="16" t="inlineStr">
         <is>
-          <t>C004_SNEHA</t>
+          <t>C004_BEHEN</t>
         </is>
       </c>
       <c r="I53" s="16" t="inlineStr">
@@ -23708,7 +23708,7 @@
       </c>
       <c r="H62" s="16" t="inlineStr">
         <is>
-          <t>A022_V_RAO</t>
+          <t>C002_ARYAN</t>
         </is>
       </c>
       <c r="I62" s="16" t="inlineStr">
@@ -23781,7 +23781,7 @@
       </c>
       <c r="H63" s="16" t="inlineStr">
         <is>
-          <t>A022_V_RAO</t>
+          <t>C002_ARYAN</t>
         </is>
       </c>
       <c r="I63" s="16" t="inlineStr">
@@ -23850,7 +23850,7 @@
       </c>
       <c r="H64" s="16" t="inlineStr">
         <is>
-          <t>A022_V_RAO</t>
+          <t>C002_ARYAN</t>
         </is>
       </c>
       <c r="I64" s="16" t="inlineStr">
@@ -23927,7 +23927,7 @@
       </c>
       <c r="H65" s="16" t="inlineStr">
         <is>
-          <t>A022_V_RAO</t>
+          <t>C002_ARYAN</t>
         </is>
       </c>
       <c r="I65" s="16" t="inlineStr">
@@ -23996,7 +23996,7 @@
       </c>
       <c r="H66" s="16" t="inlineStr">
         <is>
-          <t>A022_V_RAO</t>
+          <t>C002_ARYAN</t>
         </is>
       </c>
       <c r="I66" s="16" t="inlineStr">
@@ -24584,7 +24584,7 @@
       </c>
       <c r="H74" s="16" t="inlineStr">
         <is>
-          <t>C08-007_KAPOOR</t>
+          <t>G_M_OLD_NOGLASSES_CUT</t>
         </is>
       </c>
       <c r="I74" s="16" t="inlineStr">
@@ -24667,7 +24667,7 @@
       </c>
       <c r="H75" s="16" t="inlineStr">
         <is>
-          <t>C08-007_KAPOOR</t>
+          <t>G_M_OLD_NOGLASSES_CUT</t>
         </is>
       </c>
       <c r="I75" s="16" t="inlineStr">
@@ -24740,7 +24740,7 @@
       </c>
       <c r="H76" s="16" t="inlineStr">
         <is>
-          <t>C08-007_KAPOOR</t>
+          <t>G_M_OLD_NOGLASSES_CUT</t>
         </is>
       </c>
       <c r="I76" s="16" t="inlineStr">
@@ -24813,7 +24813,7 @@
       </c>
       <c r="H77" s="16" t="inlineStr">
         <is>
-          <t>C007_KAVYA</t>
+          <t>G_W_PINK_SUIT_CUT</t>
         </is>
       </c>
       <c r="I77" s="16" t="inlineStr">
@@ -24895,7 +24895,7 @@
       </c>
       <c r="H78" s="16" t="inlineStr">
         <is>
-          <t>C007_KAVYA</t>
+          <t>G_W_PINK_SUIT_CUT</t>
         </is>
       </c>
       <c r="I78" s="16" t="inlineStr">
@@ -24968,7 +24968,7 @@
       </c>
       <c r="H79" s="16" t="inlineStr">
         <is>
-          <t>C007_KAVYA</t>
+          <t>G_W_PINK_SUIT_CUT</t>
         </is>
       </c>
       <c r="I79" s="16" t="inlineStr">
@@ -25041,7 +25041,7 @@
       </c>
       <c r="H80" s="16" t="inlineStr">
         <is>
-          <t>G_V_MAN_CHECK_CUT</t>
+          <t>C007_VIKRAM</t>
         </is>
       </c>
       <c r="I80" s="16" t="inlineStr">
@@ -25123,7 +25123,7 @@
       </c>
       <c r="H81" s="16" t="inlineStr">
         <is>
-          <t>G_V_MAN_CHECK_CUT</t>
+          <t>C007_VIKRAM</t>
         </is>
       </c>
       <c r="I81" s="16" t="inlineStr">
@@ -25196,7 +25196,7 @@
       </c>
       <c r="H82" s="16" t="inlineStr">
         <is>
-          <t>G_V_MAN_CHECK_CUT</t>
+          <t>C007_VIKRAM</t>
         </is>
       </c>
       <c r="I82" s="16" t="inlineStr">
@@ -25269,7 +25269,7 @@
       </c>
       <c r="H83" s="16" t="inlineStr">
         <is>
-          <t>G_M_APRON_CUT</t>
+          <t>C017_CHEF</t>
         </is>
       </c>
       <c r="I83" s="16" t="inlineStr">
@@ -25352,7 +25352,7 @@
       </c>
       <c r="H84" s="16" t="inlineStr">
         <is>
-          <t>G_M_APRON_CUT</t>
+          <t>C017_CHEF</t>
         </is>
       </c>
       <c r="I84" s="16" t="inlineStr">
@@ -25425,7 +25425,7 @@
       </c>
       <c r="H85" s="16" t="inlineStr">
         <is>
-          <t>G_M_APRON_CUT</t>
+          <t>C017_CHEF</t>
         </is>
       </c>
       <c r="I85" s="16" t="inlineStr">
@@ -25498,7 +25498,7 @@
       </c>
       <c r="H86" s="16" t="inlineStr">
         <is>
-          <t>G_V_WOMAN_SAREE_CUT</t>
+          <t>C010_SUNITA</t>
         </is>
       </c>
       <c r="I86" s="16" t="inlineStr">
@@ -25581,7 +25581,7 @@
       </c>
       <c r="H87" s="16" t="inlineStr">
         <is>
-          <t>G_V_WOMAN_SAREE_CUT</t>
+          <t>C010_SUNITA</t>
         </is>
       </c>
       <c r="I87" s="16" t="inlineStr">
@@ -25654,7 +25654,7 @@
       </c>
       <c r="H88" s="16" t="inlineStr">
         <is>
-          <t>G_V_WOMAN_SAREE_CUT</t>
+          <t>C010_SUNITA</t>
         </is>
       </c>
       <c r="I88" s="16" t="inlineStr">
@@ -25727,7 +25727,7 @@
       </c>
       <c r="H89" s="16" t="inlineStr">
         <is>
-          <t>A022_JOHNNY</t>
+          <t>C015_MARCO</t>
         </is>
       </c>
       <c r="I89" s="16" t="inlineStr">
@@ -25810,7 +25810,7 @@
       </c>
       <c r="H90" s="16" t="inlineStr">
         <is>
-          <t>A022_JOHNNY</t>
+          <t>C015_MARCO</t>
         </is>
       </c>
       <c r="I90" s="16" t="inlineStr">
@@ -25883,7 +25883,7 @@
       </c>
       <c r="H91" s="16" t="inlineStr">
         <is>
-          <t>A022_JOHNNY</t>
+          <t>C015_MARCO</t>
         </is>
       </c>
       <c r="I91" s="16" t="inlineStr">
@@ -25956,7 +25956,7 @@
       </c>
       <c r="H92" s="16" t="inlineStr">
         <is>
-          <t>C04-010_ARJUN</t>
+          <t>G_M_LIGHTMAN_CUT</t>
         </is>
       </c>
       <c r="I92" s="16" t="inlineStr">
@@ -26038,7 +26038,7 @@
       </c>
       <c r="H93" s="16" t="inlineStr">
         <is>
-          <t>C04-010_ARJUN</t>
+          <t>G_M_LIGHTMAN_CUT</t>
         </is>
       </c>
       <c r="I93" s="16" t="inlineStr">
@@ -26340,7 +26340,7 @@
       </c>
       <c r="H97" s="16" t="inlineStr">
         <is>
-          <t>C005_NEHA</t>
+          <t>C018_SISTER</t>
         </is>
       </c>
       <c r="I97" s="16" t="inlineStr">
@@ -26422,7 +26422,7 @@
       </c>
       <c r="H98" s="16" t="inlineStr">
         <is>
-          <t>C005_NEHA</t>
+          <t>C018_SISTER</t>
         </is>
       </c>
       <c r="I98" s="16" t="inlineStr">
@@ -26495,7 +26495,7 @@
       </c>
       <c r="H99" s="16" t="inlineStr">
         <is>
-          <t>C005_NEHA</t>
+          <t>C018_SISTER</t>
         </is>
       </c>
       <c r="I99" s="16" t="inlineStr">
@@ -26568,7 +26568,7 @@
       </c>
       <c r="H100" s="16" t="inlineStr">
         <is>
-          <t>A022_JOHNNY</t>
+          <t>C015_MARCO</t>
         </is>
       </c>
       <c r="I100" s="16" t="inlineStr">
@@ -27175,7 +27175,7 @@
       </c>
       <c r="H108" s="16" t="inlineStr">
         <is>
-          <t>A023_V_DESHMUKH</t>
+          <t>G_V_MAN_GREY_CUT</t>
         </is>
       </c>
       <c r="I108" s="16" t="inlineStr">
@@ -27248,7 +27248,7 @@
       </c>
       <c r="H109" s="16" t="inlineStr">
         <is>
-          <t>A023_V_DESHMUKH</t>
+          <t>G_V_MAN_GREY_CUT</t>
         </is>
       </c>
       <c r="I109" s="16" t="inlineStr">
@@ -27317,7 +27317,7 @@
       </c>
       <c r="H110" s="16" t="inlineStr">
         <is>
-          <t>A023_V_DESHMUKH</t>
+          <t>G_V_MAN_GREY_CUT</t>
         </is>
       </c>
       <c r="I110" s="16" t="inlineStr">
@@ -27394,7 +27394,7 @@
       </c>
       <c r="H111" s="16" t="inlineStr">
         <is>
-          <t>A023_V_DESHMUKH</t>
+          <t>G_V_MAN_GREY_CUT</t>
         </is>
       </c>
       <c r="I111" s="16" t="inlineStr">
@@ -27463,7 +27463,7 @@
       </c>
       <c r="H112" s="16" t="inlineStr">
         <is>
-          <t>A023_V_DESHMUKH</t>
+          <t>G_V_MAN_GREY_CUT</t>
         </is>
       </c>
       <c r="I112" s="16" t="inlineStr">
@@ -27893,7 +27893,7 @@
       <c r="G118" s="16" t="inlineStr"/>
       <c r="H118" s="16" t="inlineStr">
         <is>
-          <t>P_A023_BOTTLE</t>
+          <t>P_BOTTLE_CUT</t>
         </is>
       </c>
       <c r="I118" s="16" t="inlineStr">
@@ -28280,7 +28280,7 @@
       </c>
       <c r="H123" s="16" t="inlineStr">
         <is>
-          <t>A023_BALA</t>
+          <t>C18-003_PRATEEK</t>
         </is>
       </c>
       <c r="I123" s="16" t="inlineStr">
@@ -28362,7 +28362,7 @@
       </c>
       <c r="H124" s="16" t="inlineStr">
         <is>
-          <t>A023_BALA</t>
+          <t>C18-003_PRATEEK</t>
         </is>
       </c>
       <c r="I124" s="16" t="inlineStr">
@@ -28435,7 +28435,7 @@
       </c>
       <c r="H125" s="16" t="inlineStr">
         <is>
-          <t>A023_BALA</t>
+          <t>C18-003_PRATEEK</t>
         </is>
       </c>
       <c r="I125" s="16" t="inlineStr">
@@ -28891,7 +28891,7 @@
       </c>
       <c r="H131" s="16" t="inlineStr">
         <is>
-          <t>G_V_MAN_BLUE_CUT</t>
+          <t>C020_NOAH</t>
         </is>
       </c>
       <c r="I131" s="16" t="inlineStr">
@@ -28974,7 +28974,7 @@
       </c>
       <c r="H132" s="16" t="inlineStr">
         <is>
-          <t>G_V_MAN_BLUE_CUT</t>
+          <t>C020_NOAH</t>
         </is>
       </c>
       <c r="I132" s="16" t="inlineStr">
@@ -29047,7 +29047,7 @@
       </c>
       <c r="H133" s="16" t="inlineStr">
         <is>
-          <t>G_V_MAN_BLUE_CUT</t>
+          <t>C020_NOAH</t>
         </is>
       </c>
       <c r="I133" s="16" t="inlineStr">
@@ -29120,7 +29120,7 @@
       </c>
       <c r="H134" s="16" t="inlineStr">
         <is>
-          <t>A023_ROY</t>
+          <t>G_CIVIL_RED_CUT</t>
         </is>
       </c>
       <c r="I134" s="16" t="inlineStr">
@@ -29202,7 +29202,7 @@
       </c>
       <c r="H135" s="16" t="inlineStr">
         <is>
-          <t>A023_ROY</t>
+          <t>G_CIVIL_RED_CUT</t>
         </is>
       </c>
       <c r="I135" s="16" t="inlineStr">
@@ -29275,7 +29275,7 @@
       </c>
       <c r="H136" s="16" t="inlineStr">
         <is>
-          <t>A023_ROY</t>
+          <t>G_CIVIL_RED_CUT</t>
         </is>
       </c>
       <c r="I136" s="16" t="inlineStr">
@@ -29348,7 +29348,7 @@
       </c>
       <c r="H137" s="16" t="inlineStr">
         <is>
-          <t>G_CR_VIKRAM_CUT</t>
+          <t>G_CR_MANOJ_CUT</t>
         </is>
       </c>
       <c r="I137" s="16" t="inlineStr">
@@ -29374,7 +29374,7 @@
       <c r="M137" s="16" t="inlineStr">
         <is>
           <t>SUSPECT 7/10
-Cricketer Soham
+Cricketer Manoj
 (team se nikala)</t>
         </is>
       </c>
@@ -29431,7 +29431,7 @@
       </c>
       <c r="H138" s="16" t="inlineStr">
         <is>
-          <t>G_CR_VIKRAM_CUT</t>
+          <t>G_CR_MANOJ_CUT</t>
         </is>
       </c>
       <c r="I138" s="16" t="inlineStr">
@@ -29504,7 +29504,7 @@
       </c>
       <c r="H139" s="16" t="inlineStr">
         <is>
-          <t>G_CR_VIKRAM_CUT</t>
+          <t>G_CR_MANOJ_CUT</t>
         </is>
       </c>
       <c r="I139" s="16" t="inlineStr">
@@ -29577,7 +29577,7 @@
       </c>
       <c r="H140" s="16" t="inlineStr">
         <is>
-          <t>A023_AJINKYA</t>
+          <t>G_CIVIL_GREEN_CUT</t>
         </is>
       </c>
       <c r="I140" s="16" t="inlineStr">
@@ -29659,7 +29659,7 @@
       </c>
       <c r="H141" s="16" t="inlineStr">
         <is>
-          <t>A023_AJINKYA</t>
+          <t>G_CIVIL_GREEN_CUT</t>
         </is>
       </c>
       <c r="I141" s="16" t="inlineStr">
@@ -29732,7 +29732,7 @@
       </c>
       <c r="H142" s="16" t="inlineStr">
         <is>
-          <t>A023_AJINKYA</t>
+          <t>G_CIVIL_GREEN_CUT</t>
         </is>
       </c>
       <c r="I142" s="16" t="inlineStr">
@@ -29805,7 +29805,7 @@
       </c>
       <c r="H143" s="16" t="inlineStr">
         <is>
-          <t>G_W_PINK_SUIT_CUT</t>
+          <t>A023_KAPOOR</t>
         </is>
       </c>
       <c r="I143" s="16" t="inlineStr">
@@ -29887,7 +29887,7 @@
       </c>
       <c r="H144" s="16" t="inlineStr">
         <is>
-          <t>G_W_PINK_SUIT_CUT</t>
+          <t>A023_KAPOOR</t>
         </is>
       </c>
       <c r="I144" s="16" t="inlineStr">
@@ -29960,7 +29960,7 @@
       </c>
       <c r="H145" s="16" t="inlineStr">
         <is>
-          <t>C008_NEHA</t>
+          <t>A023_SAINA</t>
         </is>
       </c>
       <c r="I145" s="16" t="inlineStr">
@@ -30042,7 +30042,7 @@
       </c>
       <c r="H146" s="16" t="inlineStr">
         <is>
-          <t>C008_NEHA</t>
+          <t>A023_SAINA</t>
         </is>
       </c>
       <c r="I146" s="16" t="inlineStr">
@@ -30722,7 +30722,7 @@
       </c>
       <c r="H155" s="16" t="inlineStr">
         <is>
-          <t>A024_V_PANDEY</t>
+          <t>C04-008_GUPTA_SLUMPED</t>
         </is>
       </c>
       <c r="I155" s="16" t="inlineStr">
@@ -30795,7 +30795,7 @@
       </c>
       <c r="H156" s="16" t="inlineStr">
         <is>
-          <t>A024_V_PANDEY</t>
+          <t>C04-008_GUPTA_SLUMPED</t>
         </is>
       </c>
       <c r="I156" s="16" t="inlineStr">
@@ -30864,7 +30864,7 @@
       </c>
       <c r="H157" s="16" t="inlineStr">
         <is>
-          <t>A024_V_PANDEY</t>
+          <t>C04-008_GUPTA_SLUMPED</t>
         </is>
       </c>
       <c r="I157" s="16" t="inlineStr">
@@ -30941,7 +30941,7 @@
       </c>
       <c r="H158" s="16" t="inlineStr">
         <is>
-          <t>A024_V_PANDEY</t>
+          <t>C04-008_GUPTA_SLUMPED</t>
         </is>
       </c>
       <c r="I158" s="16" t="inlineStr">
@@ -31010,7 +31010,7 @@
       </c>
       <c r="H159" s="16" t="inlineStr">
         <is>
-          <t>A024_V_PANDEY</t>
+          <t>C04-008_GUPTA_SLUMPED</t>
         </is>
       </c>
       <c r="I159" s="16" t="inlineStr">
@@ -31598,7 +31598,7 @@
       </c>
       <c r="H167" s="16" t="inlineStr">
         <is>
-          <t>C010_SUNITA</t>
+          <t>G_W_MAROON_SAREE_CUT</t>
         </is>
       </c>
       <c r="I167" s="16" t="inlineStr">
@@ -31681,7 +31681,7 @@
       </c>
       <c r="H168" s="16" t="inlineStr">
         <is>
-          <t>C010_SUNITA</t>
+          <t>G_W_MAROON_SAREE_CUT</t>
         </is>
       </c>
       <c r="I168" s="16" t="inlineStr">
@@ -31754,7 +31754,7 @@
       </c>
       <c r="H169" s="16" t="inlineStr">
         <is>
-          <t>C010_SUNITA</t>
+          <t>G_W_MAROON_SAREE_CUT</t>
         </is>
       </c>
       <c r="I169" s="16" t="inlineStr">
@@ -32056,7 +32056,7 @@
       </c>
       <c r="H173" s="16" t="inlineStr">
         <is>
-          <t>C004_BEHEN</t>
+          <t>C002_RIYA_CUT</t>
         </is>
       </c>
       <c r="I173" s="16" t="inlineStr">
@@ -32138,7 +32138,7 @@
       </c>
       <c r="H174" s="16" t="inlineStr">
         <is>
-          <t>C004_BEHEN</t>
+          <t>C002_RIYA_CUT</t>
         </is>
       </c>
       <c r="I174" s="16" t="inlineStr">
@@ -32211,7 +32211,7 @@
       </c>
       <c r="H175" s="16" t="inlineStr">
         <is>
-          <t>C004_BEHEN</t>
+          <t>C002_RIYA_CUT</t>
         </is>
       </c>
       <c r="I175" s="16" t="inlineStr">
@@ -32284,7 +32284,7 @@
       </c>
       <c r="H176" s="16" t="inlineStr">
         <is>
-          <t>C004_PADOSI</t>
+          <t>C12-010_MAHESH</t>
         </is>
       </c>
       <c r="I176" s="16" t="inlineStr">
@@ -32367,7 +32367,7 @@
       </c>
       <c r="H177" s="16" t="inlineStr">
         <is>
-          <t>C004_PADOSI</t>
+          <t>C12-010_MAHESH</t>
         </is>
       </c>
       <c r="I177" s="16" t="inlineStr">
@@ -32440,7 +32440,7 @@
       </c>
       <c r="H178" s="16" t="inlineStr">
         <is>
-          <t>C004_PADOSI</t>
+          <t>C12-010_MAHESH</t>
         </is>
       </c>
       <c r="I178" s="16" t="inlineStr">
@@ -32513,7 +32513,7 @@
       </c>
       <c r="H179" s="16" t="inlineStr">
         <is>
-          <t>G_V_MAN_BLUE_CUT</t>
+          <t>C003_SURAJ_CUT</t>
         </is>
       </c>
       <c r="I179" s="16" t="inlineStr">
@@ -32595,7 +32595,7 @@
       </c>
       <c r="H180" s="16" t="inlineStr">
         <is>
-          <t>G_V_MAN_BLUE_CUT</t>
+          <t>C003_SURAJ_CUT</t>
         </is>
       </c>
       <c r="I180" s="16" t="inlineStr">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H181" s="16" t="inlineStr">
         <is>
-          <t>G_V_MAN_BLUE_CUT</t>
+          <t>C003_SURAJ_CUT</t>
         </is>
       </c>
       <c r="I181" s="16" t="inlineStr">
@@ -32741,7 +32741,7 @@
       </c>
       <c r="H182" s="16" t="inlineStr">
         <is>
-          <t>G_M_YELLOW_KURTA_CUT</t>
+          <t>C001_ROHIT</t>
         </is>
       </c>
       <c r="I182" s="16" t="inlineStr">
@@ -32823,7 +32823,7 @@
       </c>
       <c r="H183" s="16" t="inlineStr">
         <is>
-          <t>G_M_YELLOW_KURTA_CUT</t>
+          <t>C001_ROHIT</t>
         </is>
       </c>
       <c r="I183" s="16" t="inlineStr">
@@ -32896,7 +32896,7 @@
       </c>
       <c r="H184" s="16" t="inlineStr">
         <is>
-          <t>G_M_YELLOW_KURTA_CUT</t>
+          <t>C001_ROHIT</t>
         </is>
       </c>
       <c r="I184" s="16" t="inlineStr">
@@ -33198,7 +33198,7 @@
       </c>
       <c r="H188" s="16" t="inlineStr">
         <is>
-          <t>G_M_LIGHTMAN_CUT</t>
+          <t>G_M_BLUE_SHIRT_CUT</t>
         </is>
       </c>
       <c r="I188" s="16" t="inlineStr">
@@ -33280,7 +33280,7 @@
       </c>
       <c r="H189" s="16" t="inlineStr">
         <is>
-          <t>G_M_LIGHTMAN_CUT</t>
+          <t>G_M_BLUE_SHIRT_CUT</t>
         </is>
       </c>
       <c r="I189" s="16" t="inlineStr">
@@ -33353,7 +33353,7 @@
       </c>
       <c r="H190" s="16" t="inlineStr">
         <is>
-          <t>G_M_LIGHTMAN_CUT</t>
+          <t>G_M_BLUE_SHIRT_CUT</t>
         </is>
       </c>
       <c r="I190" s="16" t="inlineStr">
@@ -34106,7 +34106,7 @@
       </c>
       <c r="H200" s="16" t="inlineStr">
         <is>
-          <t>A025_V_KHAN</t>
+          <t>G_V_MAN_CHECK_CUT</t>
         </is>
       </c>
       <c r="I200" s="16" t="inlineStr">
@@ -34179,7 +34179,7 @@
       </c>
       <c r="H201" s="16" t="inlineStr">
         <is>
-          <t>A025_V_KHAN</t>
+          <t>G_V_MAN_CHECK_CUT</t>
         </is>
       </c>
       <c r="I201" s="16" t="inlineStr">
@@ -34248,7 +34248,7 @@
       </c>
       <c r="H202" s="16" t="inlineStr">
         <is>
-          <t>A025_V_KHAN</t>
+          <t>G_V_MAN_CHECK_CUT</t>
         </is>
       </c>
       <c r="I202" s="16" t="inlineStr">
@@ -34325,7 +34325,7 @@
       </c>
       <c r="H203" s="16" t="inlineStr">
         <is>
-          <t>A025_V_KHAN</t>
+          <t>G_V_MAN_CHECK_CUT</t>
         </is>
       </c>
       <c r="I203" s="16" t="inlineStr">
@@ -34913,7 +34913,7 @@
       </c>
       <c r="H211" s="16" t="inlineStr">
         <is>
-          <t>C001_ROHIT</t>
+          <t>G_CR_ROHIT_CUT</t>
         </is>
       </c>
       <c r="I211" s="16" t="inlineStr">
@@ -34996,7 +34996,7 @@
       </c>
       <c r="H212" s="16" t="inlineStr">
         <is>
-          <t>C001_ROHIT</t>
+          <t>G_CR_ROHIT_CUT</t>
         </is>
       </c>
       <c r="I212" s="16" t="inlineStr">
@@ -35069,7 +35069,7 @@
       </c>
       <c r="H213" s="16" t="inlineStr">
         <is>
-          <t>C001_ROHIT</t>
+          <t>G_CR_ROHIT_CUT</t>
         </is>
       </c>
       <c r="I213" s="16" t="inlineStr">
@@ -35142,7 +35142,7 @@
       </c>
       <c r="H214" s="16" t="inlineStr">
         <is>
-          <t>G_M_BROWN_JACKET_CUT</t>
+          <t>G_M_CAMERA_CUT</t>
         </is>
       </c>
       <c r="I214" s="16" t="inlineStr">
@@ -35224,7 +35224,7 @@
       </c>
       <c r="H215" s="16" t="inlineStr">
         <is>
-          <t>G_M_BROWN_JACKET_CUT</t>
+          <t>G_M_CAMERA_CUT</t>
         </is>
       </c>
       <c r="I215" s="16" t="inlineStr">
@@ -35297,7 +35297,7 @@
       </c>
       <c r="H216" s="16" t="inlineStr">
         <is>
-          <t>G_M_BROWN_JACKET_CUT</t>
+          <t>G_M_CAMERA_CUT</t>
         </is>
       </c>
       <c r="I216" s="16" t="inlineStr">
@@ -35370,7 +35370,7 @@
       </c>
       <c r="H217" s="16" t="inlineStr">
         <is>
-          <t>C004_SNEHA</t>
+          <t>C002_POOJA</t>
         </is>
       </c>
       <c r="I217" s="16" t="inlineStr">
@@ -35453,7 +35453,7 @@
       </c>
       <c r="H218" s="16" t="inlineStr">
         <is>
-          <t>C004_SNEHA</t>
+          <t>C002_POOJA</t>
         </is>
       </c>
       <c r="I218" s="16" t="inlineStr">
@@ -35526,7 +35526,7 @@
       </c>
       <c r="H219" s="16" t="inlineStr">
         <is>
-          <t>C004_SNEHA</t>
+          <t>C002_POOJA</t>
         </is>
       </c>
       <c r="I219" s="16" t="inlineStr">
@@ -35599,7 +35599,7 @@
       </c>
       <c r="H220" s="16" t="inlineStr">
         <is>
-          <t>A025_BHUPENDRA</t>
+          <t>G_KALLU_CUT</t>
         </is>
       </c>
       <c r="I220" s="16" t="inlineStr">
@@ -35625,7 +35625,7 @@
       <c r="M220" s="16" t="inlineStr">
         <is>
           <t>SUSPECT 4/9
-Guide Bhupendra</t>
+Guide Kallu</t>
         </is>
       </c>
       <c r="N220" s="16" t="inlineStr">
@@ -35681,7 +35681,7 @@
       </c>
       <c r="H221" s="16" t="inlineStr">
         <is>
-          <t>A025_BHUPENDRA</t>
+          <t>G_KALLU_CUT</t>
         </is>
       </c>
       <c r="I221" s="16" t="inlineStr">
@@ -35754,7 +35754,7 @@
       </c>
       <c r="H222" s="16" t="inlineStr">
         <is>
-          <t>A025_BHUPENDRA</t>
+          <t>G_KALLU_CUT</t>
         </is>
       </c>
       <c r="I222" s="16" t="inlineStr">
@@ -35827,7 +35827,7 @@
       </c>
       <c r="H223" s="16" t="inlineStr">
         <is>
-          <t>C001_ANJALI</t>
+          <t>C011_EMMA</t>
         </is>
       </c>
       <c r="I223" s="16" t="inlineStr">
@@ -35909,7 +35909,7 @@
       </c>
       <c r="H224" s="16" t="inlineStr">
         <is>
-          <t>C001_ANJALI</t>
+          <t>C011_EMMA</t>
         </is>
       </c>
       <c r="I224" s="16" t="inlineStr">
@@ -35982,7 +35982,7 @@
       </c>
       <c r="H225" s="16" t="inlineStr">
         <is>
-          <t>G_V_MAN_SHERWANI_CUT</t>
+          <t>C013_LAWYER</t>
         </is>
       </c>
       <c r="I225" s="16" t="inlineStr">
@@ -36065,7 +36065,7 @@
       </c>
       <c r="H226" s="16" t="inlineStr">
         <is>
-          <t>G_V_MAN_SHERWANI_CUT</t>
+          <t>C013_LAWYER</t>
         </is>
       </c>
       <c r="I226" s="16" t="inlineStr">
@@ -36677,7 +36677,7 @@
       </c>
       <c r="H234" s="16" t="inlineStr">
         <is>
-          <t>C001_ROHIT</t>
+          <t>G_CR_ROHIT_CUT</t>
         </is>
       </c>
       <c r="I234" s="16" t="inlineStr">
@@ -37284,7 +37284,7 @@
       </c>
       <c r="H242" s="16" t="inlineStr">
         <is>
-          <t>A026_V_TSERING</t>
+          <t>C001_VIKAS</t>
         </is>
       </c>
       <c r="I242" s="16" t="inlineStr">
@@ -37357,7 +37357,7 @@
       </c>
       <c r="H243" s="16" t="inlineStr">
         <is>
-          <t>A026_V_TSERING</t>
+          <t>C001_VIKAS</t>
         </is>
       </c>
       <c r="I243" s="16" t="inlineStr">
@@ -37426,7 +37426,7 @@
       </c>
       <c r="H244" s="16" t="inlineStr">
         <is>
-          <t>A026_V_TSERING</t>
+          <t>C001_VIKAS</t>
         </is>
       </c>
       <c r="I244" s="16" t="inlineStr">
@@ -37503,7 +37503,7 @@
       </c>
       <c r="H245" s="16" t="inlineStr">
         <is>
-          <t>A026_V_TSERING</t>
+          <t>C001_VIKAS</t>
         </is>
       </c>
       <c r="I245" s="16" t="inlineStr">
@@ -37933,7 +37933,7 @@
       <c r="G251" s="16" t="inlineStr"/>
       <c r="H251" s="16" t="inlineStr">
         <is>
-          <t>P_A026_SHOES</t>
+          <t>P_SHOES</t>
         </is>
       </c>
       <c r="I251" s="16" t="inlineStr">
@@ -38320,7 +38320,7 @@
       </c>
       <c r="H256" s="16" t="inlineStr">
         <is>
-          <t>C008_NEHA</t>
+          <t>G_TANVI</t>
         </is>
       </c>
       <c r="I256" s="16" t="inlineStr">
@@ -38346,7 +38346,7 @@
       <c r="M256" s="16" t="inlineStr">
         <is>
           <t>SUSPECT 2/9
-Blogger Neha</t>
+Blogger Tanvi</t>
         </is>
       </c>
       <c r="N256" s="16" t="inlineStr">
@@ -38402,7 +38402,7 @@
       </c>
       <c r="H257" s="16" t="inlineStr">
         <is>
-          <t>C008_NEHA</t>
+          <t>G_TANVI</t>
         </is>
       </c>
       <c r="I257" s="16" t="inlineStr">
@@ -38475,7 +38475,7 @@
       </c>
       <c r="H258" s="16" t="inlineStr">
         <is>
-          <t>C008_NEHA</t>
+          <t>G_TANVI</t>
         </is>
       </c>
       <c r="I258" s="16" t="inlineStr">
@@ -38548,7 +38548,7 @@
       </c>
       <c r="H259" s="16" t="inlineStr">
         <is>
-          <t>G_M_CAMERA_CUT</t>
+          <t>G_M_BROWN_JACKET_CUT</t>
         </is>
       </c>
       <c r="I259" s="16" t="inlineStr">
@@ -38630,7 +38630,7 @@
       </c>
       <c r="H260" s="16" t="inlineStr">
         <is>
-          <t>G_M_CAMERA_CUT</t>
+          <t>G_M_BROWN_JACKET_CUT</t>
         </is>
       </c>
       <c r="I260" s="16" t="inlineStr">
@@ -38703,7 +38703,7 @@
       </c>
       <c r="H261" s="16" t="inlineStr">
         <is>
-          <t>A026_KARMA</t>
+          <t>G_M_BLUE_JACKET_B_CUT</t>
         </is>
       </c>
       <c r="I261" s="16" t="inlineStr">
@@ -38786,7 +38786,7 @@
       </c>
       <c r="H262" s="16" t="inlineStr">
         <is>
-          <t>A026_KARMA</t>
+          <t>G_M_BLUE_JACKET_B_CUT</t>
         </is>
       </c>
       <c r="I262" s="16" t="inlineStr">
@@ -38859,7 +38859,7 @@
       </c>
       <c r="H263" s="16" t="inlineStr">
         <is>
-          <t>A026_KARMA</t>
+          <t>G_M_BLUE_JACKET_B_CUT</t>
         </is>
       </c>
       <c r="I263" s="16" t="inlineStr">
@@ -38932,7 +38932,7 @@
       </c>
       <c r="H264" s="16" t="inlineStr">
         <is>
-          <t>G_M_OLD_GLASSES_CUT</t>
+          <t>C006_GUPTA</t>
         </is>
       </c>
       <c r="I264" s="16" t="inlineStr">
@@ -39014,7 +39014,7 @@
       </c>
       <c r="H265" s="16" t="inlineStr">
         <is>
-          <t>G_M_OLD_GLASSES_CUT</t>
+          <t>C006_GUPTA</t>
         </is>
       </c>
       <c r="I265" s="16" t="inlineStr">
@@ -39087,7 +39087,7 @@
       </c>
       <c r="H266" s="16" t="inlineStr">
         <is>
-          <t>C002_RIYA_CUT</t>
+          <t>C001_ANJALI</t>
         </is>
       </c>
       <c r="I266" s="16" t="inlineStr">
@@ -39169,7 +39169,7 @@
       </c>
       <c r="H267" s="16" t="inlineStr">
         <is>
-          <t>C002_RIYA_CUT</t>
+          <t>C001_ANJALI</t>
         </is>
       </c>
       <c r="I267" s="16" t="inlineStr">
@@ -39242,7 +39242,7 @@
       </c>
       <c r="H268" s="16" t="inlineStr">
         <is>
-          <t>C002_RIYA_CUT</t>
+          <t>C001_ANJALI</t>
         </is>
       </c>
       <c r="I268" s="16" t="inlineStr">
@@ -39315,7 +39315,7 @@
       </c>
       <c r="H269" s="16" t="inlineStr">
         <is>
-          <t>C16-001_DRMEHTA</t>
+          <t>G_M_OLD_GLASSES_CUT</t>
         </is>
       </c>
       <c r="I269" s="16" t="inlineStr">
@@ -39398,7 +39398,7 @@
       </c>
       <c r="H270" s="16" t="inlineStr">
         <is>
-          <t>C16-001_DRMEHTA</t>
+          <t>G_M_OLD_GLASSES_CUT</t>
         </is>
       </c>
       <c r="I270" s="16" t="inlineStr">
@@ -39471,7 +39471,7 @@
       </c>
       <c r="H271" s="16" t="inlineStr">
         <is>
-          <t>C16-001_DRMEHTA</t>
+          <t>G_M_OLD_GLASSES_CUT</t>
         </is>
       </c>
       <c r="I271" s="16" t="inlineStr">
@@ -39544,7 +39544,7 @@
       </c>
       <c r="H272" s="16" t="inlineStr">
         <is>
-          <t>A026_DORJEE</t>
+          <t>G_M_APRON_CUT</t>
         </is>
       </c>
       <c r="I272" s="16" t="inlineStr">
@@ -39627,7 +39627,7 @@
       </c>
       <c r="H273" s="16" t="inlineStr">
         <is>
-          <t>A026_DORJEE</t>
+          <t>G_M_APRON_CUT</t>
         </is>
       </c>
       <c r="I273" s="16" t="inlineStr">
@@ -39700,7 +39700,7 @@
       </c>
       <c r="H274" s="16" t="inlineStr">
         <is>
-          <t>A026_DORJEE</t>
+          <t>G_M_APRON_CUT</t>
         </is>
       </c>
       <c r="I274" s="16" t="inlineStr">
@@ -39773,7 +39773,7 @@
       </c>
       <c r="H275" s="16" t="inlineStr">
         <is>
-          <t>C007_VIKRAM</t>
+          <t>G_CIVIL_BLACK_CUT</t>
         </is>
       </c>
       <c r="I275" s="16" t="inlineStr">
@@ -39855,7 +39855,7 @@
       </c>
       <c r="H276" s="16" t="inlineStr">
         <is>
-          <t>C007_VIKRAM</t>
+          <t>G_CIVIL_BLACK_CUT</t>
         </is>
       </c>
       <c r="I276" s="16" t="inlineStr">
@@ -39928,7 +39928,7 @@
       </c>
       <c r="H277" s="16" t="inlineStr">
         <is>
-          <t>C007_VIKRAM</t>
+          <t>G_CIVIL_BLACK_CUT</t>
         </is>
       </c>
       <c r="I277" s="16" t="inlineStr">
@@ -40001,7 +40001,7 @@
       </c>
       <c r="H278" s="16" t="inlineStr">
         <is>
-          <t>A026_DORJEE</t>
+          <t>G_M_APRON_CUT</t>
         </is>
       </c>
       <c r="I278" s="16" t="inlineStr">
@@ -40074,7 +40074,7 @@
       </c>
       <c r="H279" s="16" t="inlineStr">
         <is>
-          <t>A026_DORJEE</t>
+          <t>G_M_APRON_CUT</t>
         </is>
       </c>
       <c r="I279" s="16" t="inlineStr">
@@ -40681,7 +40681,7 @@
       </c>
       <c r="H287" s="16" t="inlineStr">
         <is>
-          <t>A027_V_MOHAPATRA</t>
+          <t>G_V_MAN_SHERWANI_CUT</t>
         </is>
       </c>
       <c r="I287" s="16" t="inlineStr">
@@ -40754,7 +40754,7 @@
       </c>
       <c r="H288" s="16" t="inlineStr">
         <is>
-          <t>A027_V_MOHAPATRA</t>
+          <t>G_V_MAN_SHERWANI_CUT</t>
         </is>
       </c>
       <c r="I288" s="16" t="inlineStr">
@@ -40823,7 +40823,7 @@
       </c>
       <c r="H289" s="16" t="inlineStr">
         <is>
-          <t>A027_V_MOHAPATRA</t>
+          <t>G_V_MAN_SHERWANI_CUT</t>
         </is>
       </c>
       <c r="I289" s="16" t="inlineStr">
@@ -40900,7 +40900,7 @@
       </c>
       <c r="H290" s="16" t="inlineStr">
         <is>
-          <t>A027_V_MOHAPATRA</t>
+          <t>G_V_MAN_SHERWANI_CUT</t>
         </is>
       </c>
       <c r="I290" s="16" t="inlineStr">
@@ -40969,7 +40969,7 @@
       </c>
       <c r="H291" s="16" t="inlineStr">
         <is>
-          <t>A027_V_MOHAPATRA</t>
+          <t>G_V_MAN_SHERWANI_CUT</t>
         </is>
       </c>
       <c r="I291" s="16" t="inlineStr">
@@ -41557,7 +41557,7 @@
       </c>
       <c r="H299" s="16" t="inlineStr">
         <is>
-          <t>C002_POOJA</t>
+          <t>C019_COWORKER</t>
         </is>
       </c>
       <c r="I299" s="16" t="inlineStr">
@@ -41640,7 +41640,7 @@
       </c>
       <c r="H300" s="16" t="inlineStr">
         <is>
-          <t>C002_POOJA</t>
+          <t>C019_COWORKER</t>
         </is>
       </c>
       <c r="I300" s="16" t="inlineStr">
@@ -41713,7 +41713,7 @@
       </c>
       <c r="H301" s="16" t="inlineStr">
         <is>
-          <t>C002_POOJA</t>
+          <t>C019_COWORKER</t>
         </is>
       </c>
       <c r="I301" s="16" t="inlineStr">
@@ -41942,7 +41942,7 @@
       </c>
       <c r="H304" s="16" t="inlineStr">
         <is>
-          <t>C18-003_PRATEEK</t>
+          <t>C10-004_DEEPAK</t>
         </is>
       </c>
       <c r="I304" s="16" t="inlineStr">
@@ -42024,7 +42024,7 @@
       </c>
       <c r="H305" s="16" t="inlineStr">
         <is>
-          <t>C18-003_PRATEEK</t>
+          <t>C10-004_DEEPAK</t>
         </is>
       </c>
       <c r="I305" s="16" t="inlineStr">
@@ -42097,7 +42097,7 @@
       </c>
       <c r="H306" s="16" t="inlineStr">
         <is>
-          <t>C18-003_PRATEEK</t>
+          <t>C10-004_DEEPAK</t>
         </is>
       </c>
       <c r="I306" s="16" t="inlineStr">
@@ -42170,7 +42170,7 @@
       </c>
       <c r="H307" s="16" t="inlineStr">
         <is>
-          <t>C17-001_SETH</t>
+          <t>C017_BESTMAN</t>
         </is>
       </c>
       <c r="I307" s="16" t="inlineStr">
@@ -42252,7 +42252,7 @@
       </c>
       <c r="H308" s="16" t="inlineStr">
         <is>
-          <t>C17-001_SETH</t>
+          <t>C017_BESTMAN</t>
         </is>
       </c>
       <c r="I308" s="16" t="inlineStr">
@@ -42325,7 +42325,7 @@
       </c>
       <c r="H309" s="16" t="inlineStr">
         <is>
-          <t>C17-001_SETH</t>
+          <t>C017_BESTMAN</t>
         </is>
       </c>
       <c r="I309" s="16" t="inlineStr">
@@ -42398,7 +42398,7 @@
       </c>
       <c r="H310" s="16" t="inlineStr">
         <is>
-          <t>G_V_WOMAN_SAREE_CUT</t>
+          <t>C010_SUNITA</t>
         </is>
       </c>
       <c r="I310" s="16" t="inlineStr">
@@ -42481,7 +42481,7 @@
       </c>
       <c r="H311" s="16" t="inlineStr">
         <is>
-          <t>G_V_WOMAN_SAREE_CUT</t>
+          <t>C010_SUNITA</t>
         </is>
       </c>
       <c r="I311" s="16" t="inlineStr">
@@ -42554,7 +42554,7 @@
       </c>
       <c r="H312" s="16" t="inlineStr">
         <is>
-          <t>G_V_WOMAN_SAREE_CUT</t>
+          <t>C010_SUNITA</t>
         </is>
       </c>
       <c r="I312" s="16" t="inlineStr">
@@ -42627,7 +42627,7 @@
       </c>
       <c r="H313" s="16" t="inlineStr">
         <is>
-          <t>G_V_MAN_CHECK_CUT</t>
+          <t>C005_VICKY</t>
         </is>
       </c>
       <c r="I313" s="16" t="inlineStr">
@@ -42709,7 +42709,7 @@
       </c>
       <c r="H314" s="16" t="inlineStr">
         <is>
-          <t>G_V_MAN_CHECK_CUT</t>
+          <t>C005_VICKY</t>
         </is>
       </c>
       <c r="I314" s="16" t="inlineStr">
@@ -42782,7 +42782,7 @@
       </c>
       <c r="H315" s="16" t="inlineStr">
         <is>
-          <t>G_V_MAN_CHECK_CUT</t>
+          <t>C005_VICKY</t>
         </is>
       </c>
       <c r="I315" s="16" t="inlineStr">
@@ -42855,7 +42855,7 @@
       </c>
       <c r="H316" s="16" t="inlineStr">
         <is>
-          <t>C007_KAVYA</t>
+          <t>C004_BEHEN</t>
         </is>
       </c>
       <c r="I316" s="16" t="inlineStr">
@@ -42938,7 +42938,7 @@
       </c>
       <c r="H317" s="16" t="inlineStr">
         <is>
-          <t>C007_KAVYA</t>
+          <t>C004_BEHEN</t>
         </is>
       </c>
       <c r="I317" s="16" t="inlineStr">
@@ -43011,7 +43011,7 @@
       </c>
       <c r="H318" s="16" t="inlineStr">
         <is>
-          <t>C007_KAVYA</t>
+          <t>C004_BEHEN</t>
         </is>
       </c>
       <c r="I318" s="16" t="inlineStr">
@@ -43084,7 +43084,7 @@
       </c>
       <c r="H319" s="16" t="inlineStr">
         <is>
-          <t>G_V_MAN_GREY_CUT</t>
+          <t>C007_NIKHIL</t>
         </is>
       </c>
       <c r="I319" s="16" t="inlineStr">
@@ -43166,7 +43166,7 @@
       </c>
       <c r="H320" s="16" t="inlineStr">
         <is>
-          <t>G_V_MAN_GREY_CUT</t>
+          <t>C007_NIKHIL</t>
         </is>
       </c>
       <c r="I320" s="16" t="inlineStr">
@@ -43239,7 +43239,7 @@
       </c>
       <c r="H321" s="16" t="inlineStr">
         <is>
-          <t>G_V_MAN_GREY_CUT</t>
+          <t>C007_NIKHIL</t>
         </is>
       </c>
       <c r="I321" s="16" t="inlineStr">
@@ -43541,7 +43541,7 @@
       </c>
       <c r="H325" s="16" t="inlineStr">
         <is>
-          <t>G_RAMU</t>
+          <t>G_M_GAMCHHA_CUT</t>
         </is>
       </c>
       <c r="I325" s="16" t="inlineStr">
@@ -43567,7 +43567,7 @@
       <c r="M325" s="16" t="inlineStr">
         <is>
           <t>SUSPECT 10/10
-Safaiwala Ramu</t>
+Safaiwala Gopi</t>
         </is>
       </c>
       <c r="N325" s="16" t="inlineStr">
@@ -43623,7 +43623,7 @@
       </c>
       <c r="H326" s="16" t="inlineStr">
         <is>
-          <t>G_RAMU</t>
+          <t>G_M_GAMCHHA_CUT</t>
         </is>
       </c>
       <c r="I326" s="16" t="inlineStr">
@@ -44303,7 +44303,7 @@
       </c>
       <c r="H335" s="16" t="inlineStr">
         <is>
-          <t>A028_V_GREWAL</t>
+          <t>C08-007_KAPOOR</t>
         </is>
       </c>
       <c r="I335" s="16" t="inlineStr">
@@ -44376,7 +44376,7 @@
       </c>
       <c r="H336" s="16" t="inlineStr">
         <is>
-          <t>A028_V_GREWAL</t>
+          <t>C08-007_KAPOOR</t>
         </is>
       </c>
       <c r="I336" s="16" t="inlineStr">
@@ -44445,7 +44445,7 @@
       </c>
       <c r="H337" s="16" t="inlineStr">
         <is>
-          <t>A028_V_GREWAL</t>
+          <t>C08-007_KAPOOR</t>
         </is>
       </c>
       <c r="I337" s="16" t="inlineStr">
@@ -44522,7 +44522,7 @@
       </c>
       <c r="H338" s="16" t="inlineStr">
         <is>
-          <t>A028_V_GREWAL</t>
+          <t>C08-007_KAPOOR</t>
         </is>
       </c>
       <c r="I338" s="16" t="inlineStr">
@@ -44591,7 +44591,7 @@
       </c>
       <c r="H339" s="16" t="inlineStr">
         <is>
-          <t>A028_V_GREWAL</t>
+          <t>C08-007_KAPOOR</t>
         </is>
       </c>
       <c r="I339" s="16" t="inlineStr">
@@ -45179,7 +45179,7 @@
       </c>
       <c r="H347" s="16" t="inlineStr">
         <is>
-          <t>C005_VICKY</t>
+          <t>C018_BOYFRIEND</t>
         </is>
       </c>
       <c r="I347" s="16" t="inlineStr">
@@ -45262,7 +45262,7 @@
       </c>
       <c r="H348" s="16" t="inlineStr">
         <is>
-          <t>C005_VICKY</t>
+          <t>C018_BOYFRIEND</t>
         </is>
       </c>
       <c r="I348" s="16" t="inlineStr">
@@ -45335,7 +45335,7 @@
       </c>
       <c r="H349" s="16" t="inlineStr">
         <is>
-          <t>C005_VICKY</t>
+          <t>C018_BOYFRIEND</t>
         </is>
       </c>
       <c r="I349" s="16" t="inlineStr">
@@ -45408,7 +45408,7 @@
       </c>
       <c r="H350" s="16" t="inlineStr">
         <is>
-          <t>C005_VICKY</t>
+          <t>C018_BOYFRIEND</t>
         </is>
       </c>
       <c r="I350" s="16" t="inlineStr">
@@ -46997,7 +46997,7 @@
       </c>
       <c r="H371" s="16" t="inlineStr">
         <is>
-          <t>C001_ANJALI</t>
+          <t>A028_ANU</t>
         </is>
       </c>
       <c r="I371" s="16" t="inlineStr">
@@ -47079,7 +47079,7 @@
       </c>
       <c r="H372" s="16" t="inlineStr">
         <is>
-          <t>C001_ANJALI</t>
+          <t>A028_ANU</t>
         </is>
       </c>
       <c r="I372" s="16" t="inlineStr">
@@ -47152,7 +47152,7 @@
       </c>
       <c r="H373" s="16" t="inlineStr">
         <is>
-          <t>C001_ANJALI</t>
+          <t>A028_ANU</t>
         </is>
       </c>
       <c r="I373" s="16" t="inlineStr">
@@ -47901,7 +47901,7 @@
       </c>
       <c r="H383" s="16" t="inlineStr">
         <is>
-          <t>C04-008_GUPTA_SLUMPED</t>
+          <t>C17-001_SETH</t>
         </is>
       </c>
       <c r="I383" s="16" t="inlineStr">
@@ -47974,7 +47974,7 @@
       </c>
       <c r="H384" s="16" t="inlineStr">
         <is>
-          <t>C04-008_GUPTA_SLUMPED</t>
+          <t>C17-001_SETH</t>
         </is>
       </c>
       <c r="I384" s="16" t="inlineStr">
@@ -48043,7 +48043,7 @@
       </c>
       <c r="H385" s="16" t="inlineStr">
         <is>
-          <t>C04-008_GUPTA_SLUMPED</t>
+          <t>C17-001_SETH</t>
         </is>
       </c>
       <c r="I385" s="16" t="inlineStr">
@@ -48639,7 +48639,7 @@
       </c>
       <c r="H393" s="16" t="inlineStr">
         <is>
-          <t>C006_GUPTA</t>
+          <t>G_M_OLD_NOGLASSES_CUT</t>
         </is>
       </c>
       <c r="I393" s="16" t="inlineStr">
@@ -48721,7 +48721,7 @@
       </c>
       <c r="H394" s="16" t="inlineStr">
         <is>
-          <t>C006_GUPTA</t>
+          <t>G_M_OLD_NOGLASSES_CUT</t>
         </is>
       </c>
       <c r="I394" s="16" t="inlineStr">
@@ -48794,7 +48794,7 @@
       </c>
       <c r="H395" s="16" t="inlineStr">
         <is>
-          <t>C006_GUPTA</t>
+          <t>G_M_OLD_NOGLASSES_CUT</t>
         </is>
       </c>
       <c r="I395" s="16" t="inlineStr">
@@ -48867,7 +48867,7 @@
       </c>
       <c r="H396" s="16" t="inlineStr">
         <is>
-          <t>C006_GUPTA</t>
+          <t>G_M_OLD_NOGLASSES_CUT</t>
         </is>
       </c>
       <c r="I396" s="16" t="inlineStr">
@@ -48940,7 +48940,7 @@
       </c>
       <c r="H397" s="16" t="inlineStr">
         <is>
-          <t>C004_AMIT</t>
+          <t>C003_BHATIJA</t>
         </is>
       </c>
       <c r="I397" s="16" t="inlineStr">
@@ -49023,7 +49023,7 @@
       </c>
       <c r="H398" s="16" t="inlineStr">
         <is>
-          <t>C004_AMIT</t>
+          <t>C003_BHATIJA</t>
         </is>
       </c>
       <c r="I398" s="16" t="inlineStr">
@@ -49096,7 +49096,7 @@
       </c>
       <c r="H399" s="16" t="inlineStr">
         <is>
-          <t>C004_AMIT</t>
+          <t>C003_BHATIJA</t>
         </is>
       </c>
       <c r="I399" s="16" t="inlineStr">
@@ -49169,7 +49169,7 @@
       </c>
       <c r="H400" s="16" t="inlineStr">
         <is>
-          <t>C004_SNEHA</t>
+          <t>C002_POOJA</t>
         </is>
       </c>
       <c r="I400" s="16" t="inlineStr">
@@ -49251,7 +49251,7 @@
       </c>
       <c r="H401" s="16" t="inlineStr">
         <is>
-          <t>C004_SNEHA</t>
+          <t>C002_POOJA</t>
         </is>
       </c>
       <c r="I401" s="16" t="inlineStr">
@@ -49324,7 +49324,7 @@
       </c>
       <c r="H402" s="16" t="inlineStr">
         <is>
-          <t>C004_SNEHA</t>
+          <t>C002_POOJA</t>
         </is>
       </c>
       <c r="I402" s="16" t="inlineStr">
@@ -49397,7 +49397,7 @@
       </c>
       <c r="H403" s="16" t="inlineStr">
         <is>
-          <t>C003_BHATIJA</t>
+          <t>C004_AMIT</t>
         </is>
       </c>
       <c r="I403" s="16" t="inlineStr">
@@ -49480,7 +49480,7 @@
       </c>
       <c r="H404" s="16" t="inlineStr">
         <is>
-          <t>C003_BHATIJA</t>
+          <t>C004_AMIT</t>
         </is>
       </c>
       <c r="I404" s="16" t="inlineStr">
@@ -49553,7 +49553,7 @@
       </c>
       <c r="H405" s="16" t="inlineStr">
         <is>
-          <t>G_V_MAN_BLUE_CUT</t>
+          <t>G_M_BLUE_JACKET_A_CUT</t>
         </is>
       </c>
       <c r="I405" s="16" t="inlineStr">
@@ -49636,7 +49636,7 @@
       </c>
       <c r="H406" s="16" t="inlineStr">
         <is>
-          <t>G_V_MAN_BLUE_CUT</t>
+          <t>G_M_BLUE_JACKET_A_CUT</t>
         </is>
       </c>
       <c r="I406" s="16" t="inlineStr">
@@ -49864,7 +49864,7 @@
       </c>
       <c r="H409" s="16" t="inlineStr">
         <is>
-          <t>C08-004_MR_RATHI</t>
+          <t>C004_PADOSI</t>
         </is>
       </c>
       <c r="I409" s="16" t="inlineStr">
@@ -49947,7 +49947,7 @@
       </c>
       <c r="H410" s="16" t="inlineStr">
         <is>
-          <t>C08-004_MR_RATHI</t>
+          <t>C004_PADOSI</t>
         </is>
       </c>
       <c r="I410" s="16" t="inlineStr">
@@ -50020,7 +50020,7 @@
       </c>
       <c r="H411" s="16" t="inlineStr">
         <is>
-          <t>C08-004_MR_RATHI</t>
+          <t>C004_PADOSI</t>
         </is>
       </c>
       <c r="I411" s="16" t="inlineStr">
@@ -50403,7 +50403,7 @@
       </c>
       <c r="H416" s="16" t="inlineStr">
         <is>
-          <t>G_V_MAN_BLUE_CUT</t>
+          <t>G_M_BLUE_JACKET_A_CUT</t>
         </is>
       </c>
       <c r="I416" s="16" t="inlineStr">
@@ -51079,7 +51079,7 @@
       </c>
       <c r="H425" s="16" t="inlineStr">
         <is>
-          <t>A030_V_JOSHI</t>
+          <t>C04-010_ARJUN</t>
         </is>
       </c>
       <c r="I425" s="16" t="inlineStr">
@@ -51152,7 +51152,7 @@
       </c>
       <c r="H426" s="16" t="inlineStr">
         <is>
-          <t>A030_V_JOSHI</t>
+          <t>C04-010_ARJUN</t>
         </is>
       </c>
       <c r="I426" s="16" t="inlineStr">
@@ -51221,7 +51221,7 @@
       </c>
       <c r="H427" s="16" t="inlineStr">
         <is>
-          <t>A030_V_JOSHI</t>
+          <t>C04-010_ARJUN</t>
         </is>
       </c>
       <c r="I427" s="16" t="inlineStr">
@@ -51817,7 +51817,7 @@
       </c>
       <c r="H435" s="16" t="inlineStr">
         <is>
-          <t>G_M_GREY_HOODIE_CUT</t>
+          <t>C020_BROTHER</t>
         </is>
       </c>
       <c r="I435" s="16" t="inlineStr">
@@ -51900,7 +51900,7 @@
       </c>
       <c r="H436" s="16" t="inlineStr">
         <is>
-          <t>G_M_GREY_HOODIE_CUT</t>
+          <t>C020_BROTHER</t>
         </is>
       </c>
       <c r="I436" s="16" t="inlineStr">
@@ -51973,7 +51973,7 @@
       </c>
       <c r="H437" s="16" t="inlineStr">
         <is>
-          <t>G_M_GREY_HOODIE_CUT</t>
+          <t>C020_BROTHER</t>
         </is>
       </c>
       <c r="I437" s="16" t="inlineStr">
@@ -52046,7 +52046,7 @@
       </c>
       <c r="H438" s="16" t="inlineStr">
         <is>
-          <t>C005_NEHA</t>
+          <t>G_W_PINK_SUIT_CUT</t>
         </is>
       </c>
       <c r="I438" s="16" t="inlineStr">
@@ -52128,7 +52128,7 @@
       </c>
       <c r="H439" s="16" t="inlineStr">
         <is>
-          <t>C005_NEHA</t>
+          <t>G_W_PINK_SUIT_CUT</t>
         </is>
       </c>
       <c r="I439" s="16" t="inlineStr">
@@ -52201,7 +52201,7 @@
       </c>
       <c r="H440" s="16" t="inlineStr">
         <is>
-          <t>G_M_OLD_NOGLASSES_CUT</t>
+          <t>C011_TOM</t>
         </is>
       </c>
       <c r="I440" s="16" t="inlineStr">
@@ -52283,7 +52283,7 @@
       </c>
       <c r="H441" s="16" t="inlineStr">
         <is>
-          <t>G_M_OLD_NOGLASSES_CUT</t>
+          <t>C011_TOM</t>
         </is>
       </c>
       <c r="I441" s="16" t="inlineStr">
@@ -52356,7 +52356,7 @@
       </c>
       <c r="H442" s="16" t="inlineStr">
         <is>
-          <t>G_M_OLD_NOGLASSES_CUT</t>
+          <t>C011_TOM</t>
         </is>
       </c>
       <c r="I442" s="16" t="inlineStr">
@@ -52429,7 +52429,7 @@
       </c>
       <c r="H443" s="16" t="inlineStr">
         <is>
-          <t>C007_KAVYA</t>
+          <t>C018_SISTER</t>
         </is>
       </c>
       <c r="I443" s="16" t="inlineStr">
@@ -52512,7 +52512,7 @@
       </c>
       <c r="H444" s="16" t="inlineStr">
         <is>
-          <t>C007_KAVYA</t>
+          <t>C018_SISTER</t>
         </is>
       </c>
       <c r="I444" s="16" t="inlineStr">
@@ -52585,7 +52585,7 @@
       </c>
       <c r="H445" s="16" t="inlineStr">
         <is>
-          <t>C007_KAVYA</t>
+          <t>C018_SISTER</t>
         </is>
       </c>
       <c r="I445" s="16" t="inlineStr">
@@ -52658,7 +52658,7 @@
       </c>
       <c r="H446" s="16" t="inlineStr">
         <is>
-          <t>C007_KAVYA</t>
+          <t>C018_SISTER</t>
         </is>
       </c>
       <c r="I446" s="16" t="inlineStr">
@@ -53417,7 +53417,7 @@
       </c>
       <c r="H456" s="16" t="inlineStr">
         <is>
-          <t>C10-004_DEEPAK</t>
+          <t>C03-003_VICKY</t>
         </is>
       </c>
       <c r="I456" s="16" t="inlineStr">
@@ -53500,7 +53500,7 @@
       </c>
       <c r="H457" s="16" t="inlineStr">
         <is>
-          <t>C10-004_DEEPAK</t>
+          <t>C03-003_VICKY</t>
         </is>
       </c>
       <c r="I457" s="16" t="inlineStr">
@@ -53573,7 +53573,7 @@
       </c>
       <c r="H458" s="16" t="inlineStr">
         <is>
-          <t>C10-004_DEEPAK</t>
+          <t>C03-003_VICKY</t>
         </is>
       </c>
       <c r="I458" s="16" t="inlineStr">
@@ -53874,7 +53874,7 @@
       </c>
       <c r="H462" s="16" t="inlineStr">
         <is>
-          <t>G_V_MAN_CHECK_CUT</t>
+          <t>C008_GUEST</t>
         </is>
       </c>
       <c r="I462" s="16" t="inlineStr">
@@ -53956,7 +53956,7 @@
       </c>
       <c r="H463" s="16" t="inlineStr">
         <is>
-          <t>G_V_MAN_CHECK_CUT</t>
+          <t>C008_GUEST</t>
         </is>
       </c>
       <c r="I463" s="16" t="inlineStr">
@@ -54029,7 +54029,7 @@
       </c>
       <c r="H464" s="16" t="inlineStr">
         <is>
-          <t>G_V_MAN_CHECK_CUT</t>
+          <t>C008_GUEST</t>
         </is>
       </c>
       <c r="I464" s="16" t="inlineStr">
@@ -54102,7 +54102,7 @@
       </c>
       <c r="H465" s="16" t="inlineStr">
         <is>
-          <t>G_M_GREY_HOODIE_CUT</t>
+          <t>C020_BROTHER</t>
         </is>
       </c>
       <c r="I465" s="16" t="inlineStr">
@@ -56443,7 +56443,7 @@
       </c>
       <c r="H3" s="16" t="inlineStr">
         <is>
-          <t>A021_V_KAMLESH</t>
+          <t>C08-004_MR_RATHI</t>
         </is>
       </c>
       <c r="I3" s="16" t="inlineStr">
@@ -56516,7 +56516,7 @@
       </c>
       <c r="H4" s="16" t="inlineStr">
         <is>
-          <t>A021_V_KAMLESH</t>
+          <t>C08-004_MR_RATHI</t>
         </is>
       </c>
       <c r="I4" s="16" t="inlineStr">
@@ -56585,7 +56585,7 @@
       </c>
       <c r="H5" s="16" t="inlineStr">
         <is>
-          <t>A021_V_KAMLESH</t>
+          <t>C08-004_MR_RATHI</t>
         </is>
       </c>
       <c r="I5" s="16" t="inlineStr">
@@ -56662,7 +56662,7 @@
       </c>
       <c r="H6" s="16" t="inlineStr">
         <is>
-          <t>A021_V_KAMLESH</t>
+          <t>C08-004_MR_RATHI</t>
         </is>
       </c>
       <c r="I6" s="16" t="inlineStr">
@@ -56731,7 +56731,7 @@
       </c>
       <c r="H7" s="16" t="inlineStr">
         <is>
-          <t>A021_V_KAMLESH</t>
+          <t>C08-004_MR_RATHI</t>
         </is>
       </c>
       <c r="I7" s="16" t="inlineStr">
@@ -56873,7 +56873,7 @@
       </c>
       <c r="H9" s="16" t="inlineStr">
         <is>
-          <t>P_KAANCH_TUKDE_CUT ... P_A021_PHOTO</t>
+          <t>P_KAANCH_TUKDE ... P_A021_PHOTO</t>
         </is>
       </c>
       <c r="I9" s="16" t="inlineStr">
@@ -56950,7 +56950,7 @@
       </c>
       <c r="H10" s="16" t="inlineStr">
         <is>
-          <t>P_KAANCH_TUKDE_CUT ... P_A021_PHOTO</t>
+          <t>P_KAANCH_TUKDE ... P_A021_PHOTO</t>
         </is>
       </c>
       <c r="I10" s="16" t="inlineStr">
@@ -57023,7 +57023,7 @@
       </c>
       <c r="H11" s="16" t="inlineStr">
         <is>
-          <t>P_KAANCH_TUKDE_CUT ... P_A021_PHOTO</t>
+          <t>P_KAANCH_TUKDE ... P_A021_PHOTO</t>
         </is>
       </c>
       <c r="I11" s="16" t="inlineStr">
@@ -57481,7 +57481,7 @@
       </c>
       <c r="H17" s="16" t="inlineStr">
         <is>
-          <t>G_M_CAMERA_CUT</t>
+          <t>G_M_YELLOW_KURTA_CUT</t>
         </is>
       </c>
       <c r="I17" s="16" t="inlineStr">
@@ -57563,7 +57563,7 @@
       </c>
       <c r="H18" s="16" t="inlineStr">
         <is>
-          <t>G_M_CAMERA_CUT</t>
+          <t>G_M_YELLOW_KURTA_CUT</t>
         </is>
       </c>
       <c r="I18" s="16" t="inlineStr">
@@ -57636,7 +57636,7 @@
       </c>
       <c r="H19" s="16" t="inlineStr">
         <is>
-          <t>G_M_CAMERA_CUT</t>
+          <t>G_M_YELLOW_KURTA_CUT</t>
         </is>
       </c>
       <c r="I19" s="16" t="inlineStr">
@@ -57709,7 +57709,7 @@
       </c>
       <c r="H20" s="16" t="inlineStr">
         <is>
-          <t>G_V_MAN_GREY_CUT</t>
+          <t>C005_VICKY_KEY_CUT</t>
         </is>
       </c>
       <c r="I20" s="16" t="inlineStr">
@@ -57792,7 +57792,7 @@
       </c>
       <c r="H21" s="16" t="inlineStr">
         <is>
-          <t>G_V_MAN_GREY_CUT</t>
+          <t>C005_VICKY_KEY_CUT</t>
         </is>
       </c>
       <c r="I21" s="16" t="inlineStr">
@@ -57865,7 +57865,7 @@
       </c>
       <c r="H22" s="16" t="inlineStr">
         <is>
-          <t>C004_SNEHA</t>
+          <t>C004_BEHEN</t>
         </is>
       </c>
       <c r="I22" s="16" t="inlineStr">
@@ -57947,7 +57947,7 @@
       </c>
       <c r="H23" s="16" t="inlineStr">
         <is>
-          <t>C004_SNEHA</t>
+          <t>C004_BEHEN</t>
         </is>
       </c>
       <c r="I23" s="16" t="inlineStr">
@@ -58474,7 +58474,7 @@
       </c>
       <c r="H30" s="16" t="inlineStr">
         <is>
-          <t>A022_V_RAO</t>
+          <t>C002_ARYAN</t>
         </is>
       </c>
       <c r="I30" s="16" t="inlineStr">
@@ -58547,7 +58547,7 @@
       </c>
       <c r="H31" s="16" t="inlineStr">
         <is>
-          <t>A022_V_RAO</t>
+          <t>C002_ARYAN</t>
         </is>
       </c>
       <c r="I31" s="16" t="inlineStr">
@@ -58616,7 +58616,7 @@
       </c>
       <c r="H32" s="16" t="inlineStr">
         <is>
-          <t>A022_V_RAO</t>
+          <t>C002_ARYAN</t>
         </is>
       </c>
       <c r="I32" s="16" t="inlineStr">
@@ -58693,7 +58693,7 @@
       </c>
       <c r="H33" s="16" t="inlineStr">
         <is>
-          <t>A022_V_RAO</t>
+          <t>C002_ARYAN</t>
         </is>
       </c>
       <c r="I33" s="16" t="inlineStr">
@@ -59058,7 +59058,7 @@
       </c>
       <c r="H38" s="16" t="inlineStr">
         <is>
-          <t>C08-007_KAPOOR</t>
+          <t>G_M_OLD_NOGLASSES_CUT</t>
         </is>
       </c>
       <c r="I38" s="16" t="inlineStr">
@@ -59141,7 +59141,7 @@
       </c>
       <c r="H39" s="16" t="inlineStr">
         <is>
-          <t>C08-007_KAPOOR</t>
+          <t>G_M_OLD_NOGLASSES_CUT</t>
         </is>
       </c>
       <c r="I39" s="16" t="inlineStr">
@@ -59214,7 +59214,7 @@
       </c>
       <c r="H40" s="16" t="inlineStr">
         <is>
-          <t>G_V_MAN_CHECK_CUT</t>
+          <t>C007_VIKRAM</t>
         </is>
       </c>
       <c r="I40" s="16" t="inlineStr">
@@ -59296,7 +59296,7 @@
       </c>
       <c r="H41" s="16" t="inlineStr">
         <is>
-          <t>G_V_MAN_CHECK_CUT</t>
+          <t>C007_VIKRAM</t>
         </is>
       </c>
       <c r="I41" s="16" t="inlineStr">
@@ -59369,7 +59369,7 @@
       </c>
       <c r="H42" s="16" t="inlineStr">
         <is>
-          <t>G_V_MAN_CHECK_CUT</t>
+          <t>C007_VIKRAM</t>
         </is>
       </c>
       <c r="I42" s="16" t="inlineStr">
@@ -59442,7 +59442,7 @@
       </c>
       <c r="H43" s="16" t="inlineStr">
         <is>
-          <t>G_V_WOMAN_SAREE_CUT</t>
+          <t>C010_SUNITA</t>
         </is>
       </c>
       <c r="I43" s="16" t="inlineStr">
@@ -59525,7 +59525,7 @@
       </c>
       <c r="H44" s="16" t="inlineStr">
         <is>
-          <t>G_V_WOMAN_SAREE_CUT</t>
+          <t>C010_SUNITA</t>
         </is>
       </c>
       <c r="I44" s="16" t="inlineStr">
@@ -59598,7 +59598,7 @@
       </c>
       <c r="H45" s="16" t="inlineStr">
         <is>
-          <t>A022_JOHNNY</t>
+          <t>C015_MARCO</t>
         </is>
       </c>
       <c r="I45" s="16" t="inlineStr">
@@ -59681,7 +59681,7 @@
       </c>
       <c r="H46" s="16" t="inlineStr">
         <is>
-          <t>A022_JOHNNY</t>
+          <t>C015_MARCO</t>
         </is>
       </c>
       <c r="I46" s="16" t="inlineStr">
@@ -59754,7 +59754,7 @@
       </c>
       <c r="H47" s="16" t="inlineStr">
         <is>
-          <t>C005_NEHA</t>
+          <t>C018_SISTER</t>
         </is>
       </c>
       <c r="I47" s="16" t="inlineStr">
@@ -59836,7 +59836,7 @@
       </c>
       <c r="H48" s="16" t="inlineStr">
         <is>
-          <t>C005_NEHA</t>
+          <t>C018_SISTER</t>
         </is>
       </c>
       <c r="I48" s="16" t="inlineStr">
@@ -60363,7 +60363,7 @@
       </c>
       <c r="H55" s="16" t="inlineStr">
         <is>
-          <t>A027_V_MOHAPATRA</t>
+          <t>G_V_MAN_SHERWANI_CUT</t>
         </is>
       </c>
       <c r="I55" s="16" t="inlineStr">
@@ -60436,7 +60436,7 @@
       </c>
       <c r="H56" s="16" t="inlineStr">
         <is>
-          <t>A027_V_MOHAPATRA</t>
+          <t>G_V_MAN_SHERWANI_CUT</t>
         </is>
       </c>
       <c r="I56" s="16" t="inlineStr">
@@ -60505,7 +60505,7 @@
       </c>
       <c r="H57" s="16" t="inlineStr">
         <is>
-          <t>A027_V_MOHAPATRA</t>
+          <t>G_V_MAN_SHERWANI_CUT</t>
         </is>
       </c>
       <c r="I57" s="16" t="inlineStr">
@@ -60582,7 +60582,7 @@
       </c>
       <c r="H58" s="16" t="inlineStr">
         <is>
-          <t>A027_V_MOHAPATRA</t>
+          <t>G_V_MAN_SHERWANI_CUT</t>
         </is>
       </c>
       <c r="I58" s="16" t="inlineStr">
@@ -60947,7 +60947,7 @@
       </c>
       <c r="H63" s="16" t="inlineStr">
         <is>
-          <t>C002_POOJA</t>
+          <t>C019_COWORKER</t>
         </is>
       </c>
       <c r="I63" s="16" t="inlineStr">
@@ -61030,7 +61030,7 @@
       </c>
       <c r="H64" s="16" t="inlineStr">
         <is>
-          <t>C002_POOJA</t>
+          <t>C019_COWORKER</t>
         </is>
       </c>
       <c r="I64" s="16" t="inlineStr">
@@ -61186,7 +61186,7 @@
       </c>
       <c r="H66" s="16" t="inlineStr">
         <is>
-          <t>C17-001_SETH</t>
+          <t>C017_BESTMAN</t>
         </is>
       </c>
       <c r="I66" s="16" t="inlineStr">
@@ -61268,7 +61268,7 @@
       </c>
       <c r="H67" s="16" t="inlineStr">
         <is>
-          <t>C17-001_SETH</t>
+          <t>C017_BESTMAN</t>
         </is>
       </c>
       <c r="I67" s="16" t="inlineStr">
@@ -61341,7 +61341,7 @@
       </c>
       <c r="H68" s="16" t="inlineStr">
         <is>
-          <t>C17-001_SETH</t>
+          <t>C017_BESTMAN</t>
         </is>
       </c>
       <c r="I68" s="16" t="inlineStr">
@@ -61414,7 +61414,7 @@
       </c>
       <c r="H69" s="16" t="inlineStr">
         <is>
-          <t>C007_KAVYA</t>
+          <t>C004_BEHEN</t>
         </is>
       </c>
       <c r="I69" s="16" t="inlineStr">
@@ -61497,7 +61497,7 @@
       </c>
       <c r="H70" s="16" t="inlineStr">
         <is>
-          <t>C007_KAVYA</t>
+          <t>C004_BEHEN</t>
         </is>
       </c>
       <c r="I70" s="16" t="inlineStr">
@@ -62309,36 +62309,36 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="16" t="inlineStr">
-        <is>
-          <t>A021_V_KAMLESH</t>
-        </is>
-      </c>
-      <c r="B9" s="16" t="inlineStr">
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>C08-004_MR_RATHI</t>
+        </is>
+      </c>
+      <c r="B9" s="19" t="inlineStr">
         <is>
           <t>A021</t>
         </is>
       </c>
-      <c r="C9" s="16" t="inlineStr">
+      <c r="C9" s="19" t="inlineStr">
         <is>
           <t>Victim</t>
         </is>
       </c>
-      <c r="D9" s="16" t="inlineStr">
+      <c r="D9" s="19" t="inlineStr">
         <is>
           <t>Indian mill owner Kamlesh Agrawal, about 58, kurta and Nehru jacket, slumped on a leather chair, eyes closed</t>
         </is>
       </c>
-      <c r="E9" s="16" t="inlineStr">
-        <is>
-          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Indian mill owner Kamlesh Agrawal, about 58, kurta and Nehru jacket, slumped on a leather chair, eyes closed. Peaceful pose, YouTube-safe: no blood, no wounds. Plain bright green (#00FF00) background, no text, no shadow.</t>
+      <c r="E9" s="19" t="inlineStr">
+        <is>
+          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="19" t="inlineStr">
         <is>
-          <t>P_KAANCH_TUKDE_CUT</t>
+          <t>P_KAANCH_TUKDE</t>
         </is>
       </c>
       <c r="B10" s="19" t="inlineStr">
@@ -62554,7 +62554,7 @@
     <row r="18">
       <c r="A18" s="19" t="inlineStr">
         <is>
-          <t>G_W_MAROON_SAREE_CUT</t>
+          <t>C004_MAA</t>
         </is>
       </c>
       <c r="B18" s="19" t="inlineStr">
@@ -62581,7 +62581,7 @@
     <row r="19">
       <c r="A19" s="19" t="inlineStr">
         <is>
-          <t>G_M_CAMERA_CUT</t>
+          <t>G_M_YELLOW_KURTA_CUT</t>
         </is>
       </c>
       <c r="B19" s="19" t="inlineStr">
@@ -62608,7 +62608,7 @@
     <row r="20">
       <c r="A20" s="19" t="inlineStr">
         <is>
-          <t>G_V_MAN_GREY_CUT</t>
+          <t>C005_VICKY_KEY_CUT</t>
         </is>
       </c>
       <c r="B20" s="19" t="inlineStr">
@@ -62635,7 +62635,7 @@
     <row r="21">
       <c r="A21" s="19" t="inlineStr">
         <is>
-          <t>C08-004_MR_RATHI</t>
+          <t>G_TTE</t>
         </is>
       </c>
       <c r="B21" s="19" t="inlineStr">
@@ -62662,7 +62662,7 @@
     <row r="22">
       <c r="A22" s="19" t="inlineStr">
         <is>
-          <t>C004_SNEHA</t>
+          <t>C004_BEHEN</t>
         </is>
       </c>
       <c r="B22" s="19" t="inlineStr">
@@ -62714,29 +62714,29 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="16" t="inlineStr">
-        <is>
-          <t>A022_V_RAO</t>
-        </is>
-      </c>
-      <c r="B24" s="16" t="inlineStr">
+      <c r="A24" s="19" t="inlineStr">
+        <is>
+          <t>C002_ARYAN</t>
+        </is>
+      </c>
+      <c r="B24" s="19" t="inlineStr">
         <is>
           <t>A022</t>
         </is>
       </c>
-      <c r="C24" s="16" t="inlineStr">
+      <c r="C24" s="19" t="inlineStr">
         <is>
           <t>Victim</t>
         </is>
       </c>
-      <c r="D24" s="16" t="inlineStr">
+      <c r="D24" s="19" t="inlineStr">
         <is>
           <t>Indian resort owner Srinivas Rao, about 55, white shirt, slumped on an office chair, eyes closed</t>
         </is>
       </c>
-      <c r="E24" s="16" t="inlineStr">
-        <is>
-          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Indian resort owner Srinivas Rao, about 55, white shirt, slumped on an office chair, eyes closed. Peaceful pose, YouTube-safe: no blood, no wounds. Plain bright green (#00FF00) background, no text, no shadow.</t>
+      <c r="E24" s="19" t="inlineStr">
+        <is>
+          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
         </is>
       </c>
     </row>
@@ -62878,7 +62878,7 @@
     <row r="30">
       <c r="A30" s="19" t="inlineStr">
         <is>
-          <t>C08-007_KAPOOR</t>
+          <t>G_M_OLD_NOGLASSES_CUT</t>
         </is>
       </c>
       <c r="B30" s="19" t="inlineStr">
@@ -62905,7 +62905,7 @@
     <row r="31">
       <c r="A31" s="19" t="inlineStr">
         <is>
-          <t>C007_KAVYA</t>
+          <t>G_W_PINK_SUIT_CUT</t>
         </is>
       </c>
       <c r="B31" s="19" t="inlineStr">
@@ -62932,7 +62932,7 @@
     <row r="32">
       <c r="A32" s="19" t="inlineStr">
         <is>
-          <t>G_V_MAN_CHECK_CUT</t>
+          <t>C007_VIKRAM</t>
         </is>
       </c>
       <c r="B32" s="19" t="inlineStr">
@@ -62959,7 +62959,7 @@
     <row r="33">
       <c r="A33" s="19" t="inlineStr">
         <is>
-          <t>G_M_APRON_CUT</t>
+          <t>C017_CHEF</t>
         </is>
       </c>
       <c r="B33" s="19" t="inlineStr">
@@ -62986,7 +62986,7 @@
     <row r="34">
       <c r="A34" s="19" t="inlineStr">
         <is>
-          <t>G_V_WOMAN_SAREE_CUT</t>
+          <t>C010_SUNITA</t>
         </is>
       </c>
       <c r="B34" s="19" t="inlineStr">
@@ -63011,36 +63011,36 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="16" t="inlineStr">
-        <is>
-          <t>A022_JOHNNY</t>
-        </is>
-      </c>
-      <c r="B35" s="16" t="inlineStr">
+      <c r="A35" s="19" t="inlineStr">
+        <is>
+          <t>C015_MARCO</t>
+        </is>
+      </c>
+      <c r="B35" s="19" t="inlineStr">
         <is>
           <t>A022</t>
         </is>
       </c>
-      <c r="C35" s="16" t="inlineStr">
+      <c r="C35" s="19" t="inlineStr">
         <is>
           <t>Suspect</t>
         </is>
       </c>
-      <c r="D35" s="16" t="inlineStr">
+      <c r="D35" s="19" t="inlineStr">
         <is>
           <t>Lifeguard Johnny (geele pair isi ke)</t>
         </is>
       </c>
-      <c r="E35" s="16" t="inlineStr">
-        <is>
-          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Fit young man about 28, lifeguard vest, wet hair. Full body, standing, facing camera. Plain bright green (#00FF00) background, no text, no shadow.</t>
+      <c r="E35" s="19" t="inlineStr">
+        <is>
+          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="19" t="inlineStr">
         <is>
-          <t>C04-010_ARJUN</t>
+          <t>G_M_LIGHTMAN_CUT</t>
         </is>
       </c>
       <c r="B36" s="19" t="inlineStr">
@@ -63094,7 +63094,7 @@
     <row r="38">
       <c r="A38" s="19" t="inlineStr">
         <is>
-          <t>C005_NEHA</t>
+          <t>C018_SISTER</t>
         </is>
       </c>
       <c r="B38" s="19" t="inlineStr">
@@ -63146,29 +63146,29 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="16" t="inlineStr">
-        <is>
-          <t>A023_V_DESHMUKH</t>
-        </is>
-      </c>
-      <c r="B40" s="16" t="inlineStr">
+      <c r="A40" s="19" t="inlineStr">
+        <is>
+          <t>G_V_MAN_GREY_CUT</t>
+        </is>
+      </c>
+      <c r="B40" s="19" t="inlineStr">
         <is>
           <t>A023</t>
         </is>
       </c>
-      <c r="C40" s="16" t="inlineStr">
+      <c r="C40" s="19" t="inlineStr">
         <is>
           <t>Victim</t>
         </is>
       </c>
-      <c r="D40" s="16" t="inlineStr">
+      <c r="D40" s="19" t="inlineStr">
         <is>
           <t>Indian sports club president Vijay Deshmukh, about 60, track jacket, slumped on a locker room bench, eyes closed</t>
         </is>
       </c>
-      <c r="E40" s="16" t="inlineStr">
-        <is>
-          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Indian sports club president Vijay Deshmukh, about 60, track jacket, slumped on a locker room bench, eyes closed. Peaceful pose, YouTube-safe: no blood, no wounds. Plain bright green (#00FF00) background, no text, no shadow.</t>
+      <c r="E40" s="19" t="inlineStr">
+        <is>
+          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
         </is>
       </c>
     </row>
@@ -63281,29 +63281,29 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="18" t="inlineStr">
-        <is>
-          <t>P_A023_BOTTLE</t>
-        </is>
-      </c>
-      <c r="B45" s="18" t="inlineStr">
+      <c r="A45" s="19" t="inlineStr">
+        <is>
+          <t>P_BOTTLE_CUT</t>
+        </is>
+      </c>
+      <c r="B45" s="19" t="inlineStr">
         <is>
           <t>A023</t>
         </is>
       </c>
-      <c r="C45" s="18" t="inlineStr">
+      <c r="C45" s="19" t="inlineStr">
         <is>
           <t>Saboot (prop)</t>
         </is>
       </c>
-      <c r="D45" s="18" t="inlineStr">
+      <c r="D45" s="19" t="inlineStr">
         <is>
           <t>Spilled sports water bottle</t>
         </is>
       </c>
-      <c r="E45" s="18" t="inlineStr">
-        <is>
-          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Spilled sports water bottle. Close-up object, centered. Plain bright green (#00FF00) background, no text, no shadow.</t>
+      <c r="E45" s="19" t="inlineStr">
+        <is>
+          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
         </is>
       </c>
     </row>
@@ -63335,29 +63335,29 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="16" t="inlineStr">
-        <is>
-          <t>A023_BALA</t>
-        </is>
-      </c>
-      <c r="B47" s="16" t="inlineStr">
+      <c r="A47" s="19" t="inlineStr">
+        <is>
+          <t>C18-003_PRATEEK</t>
+        </is>
+      </c>
+      <c r="B47" s="19" t="inlineStr">
         <is>
           <t>A023</t>
         </is>
       </c>
-      <c r="C47" s="16" t="inlineStr">
+      <c r="C47" s="19" t="inlineStr">
         <is>
           <t>Suspect</t>
         </is>
       </c>
-      <c r="D47" s="16" t="inlineStr">
+      <c r="D47" s="19" t="inlineStr">
         <is>
           <t>Kabaddi khiladi Bala</t>
         </is>
       </c>
-      <c r="E47" s="16" t="inlineStr">
-        <is>
-          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Muscular young man about 25, kabaddi vest. Full body, standing, facing camera. Plain bright green (#00FF00) background, no text, no shadow.</t>
+      <c r="E47" s="19" t="inlineStr">
+        <is>
+          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
         </is>
       </c>
     </row>
@@ -63418,7 +63418,7 @@
     <row r="50">
       <c r="A50" s="19" t="inlineStr">
         <is>
-          <t>G_V_MAN_BLUE_CUT</t>
+          <t>C020_NOAH</t>
         </is>
       </c>
       <c r="B50" s="19" t="inlineStr">
@@ -63443,36 +63443,36 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="16" t="inlineStr">
-        <is>
-          <t>A023_ROY</t>
-        </is>
-      </c>
-      <c r="B51" s="16" t="inlineStr">
+      <c r="A51" s="19" t="inlineStr">
+        <is>
+          <t>G_CIVIL_RED_CUT</t>
+        </is>
+      </c>
+      <c r="B51" s="19" t="inlineStr">
         <is>
           <t>A023</t>
         </is>
       </c>
-      <c r="C51" s="16" t="inlineStr">
+      <c r="C51" s="19" t="inlineStr">
         <is>
           <t>Suspect</t>
         </is>
       </c>
-      <c r="D51" s="16" t="inlineStr">
+      <c r="D51" s="19" t="inlineStr">
         <is>
           <t>Basketball coach Roy</t>
         </is>
       </c>
-      <c r="E51" s="16" t="inlineStr">
-        <is>
-          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Tall Indian man about 38, basketball jersey. Full body, standing, facing camera. Plain bright green (#00FF00) background, no text, no shadow.</t>
+      <c r="E51" s="19" t="inlineStr">
+        <is>
+          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="19" t="inlineStr">
         <is>
-          <t>G_CR_VIKRAM_CUT</t>
+          <t>G_CR_MANOJ_CUT</t>
         </is>
       </c>
       <c r="B52" s="19" t="inlineStr">
@@ -63487,7 +63487,7 @@
       </c>
       <c r="D52" s="19" t="inlineStr">
         <is>
-          <t>Cricketer Soham (team se nikala)</t>
+          <t>Cricketer Manoj (team se nikala)</t>
         </is>
       </c>
       <c r="E52" s="19" t="inlineStr">
@@ -63497,83 +63497,83 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="16" t="inlineStr">
-        <is>
-          <t>A023_AJINKYA</t>
-        </is>
-      </c>
-      <c r="B53" s="16" t="inlineStr">
+      <c r="A53" s="19" t="inlineStr">
+        <is>
+          <t>G_CIVIL_GREEN_CUT</t>
+        </is>
+      </c>
+      <c r="B53" s="19" t="inlineStr">
         <is>
           <t>A023</t>
         </is>
       </c>
-      <c r="C53" s="16" t="inlineStr">
+      <c r="C53" s="19" t="inlineStr">
         <is>
           <t>Suspect</t>
         </is>
       </c>
-      <c r="D53" s="16" t="inlineStr">
+      <c r="D53" s="19" t="inlineStr">
         <is>
           <t>Volleyball captain Ajinkya</t>
         </is>
       </c>
-      <c r="E53" s="16" t="inlineStr">
-        <is>
-          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Tall young man about 26, volleyball jersey, ball, confident. Full body, standing, facing camera. Plain bright green (#00FF00) background, no text, no shadow.</t>
+      <c r="E53" s="19" t="inlineStr">
+        <is>
+          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="19" t="inlineStr">
-        <is>
-          <t>G_W_PINK_SUIT_CUT</t>
-        </is>
-      </c>
-      <c r="B54" s="19" t="inlineStr">
+      <c r="A54" s="16" t="inlineStr">
+        <is>
+          <t>A023_KAPOOR</t>
+        </is>
+      </c>
+      <c r="B54" s="16" t="inlineStr">
         <is>
           <t>A023</t>
         </is>
       </c>
-      <c r="C54" s="19" t="inlineStr">
+      <c r="C54" s="16" t="inlineStr">
         <is>
           <t>Suspect</t>
         </is>
       </c>
-      <c r="D54" s="19" t="inlineStr">
+      <c r="D54" s="16" t="inlineStr">
         <is>
           <t>Golfer Mrs. Kapoor</t>
         </is>
       </c>
-      <c r="E54" s="19" t="inlineStr">
-        <is>
-          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
+      <c r="E54" s="16" t="inlineStr">
+        <is>
+          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Indian woman about 50, golf cap, golf club. Full body, standing, facing camera. Plain bright green (#00FF00) background, no text, no shadow.</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="19" t="inlineStr">
-        <is>
-          <t>C008_NEHA</t>
-        </is>
-      </c>
-      <c r="B55" s="19" t="inlineStr">
+      <c r="A55" s="16" t="inlineStr">
+        <is>
+          <t>A023_SAINA</t>
+        </is>
+      </c>
+      <c r="B55" s="16" t="inlineStr">
         <is>
           <t>A023</t>
         </is>
       </c>
-      <c r="C55" s="19" t="inlineStr">
+      <c r="C55" s="16" t="inlineStr">
         <is>
           <t>Suspect</t>
         </is>
       </c>
-      <c r="D55" s="19" t="inlineStr">
+      <c r="D55" s="16" t="inlineStr">
         <is>
           <t>Badminton khiladi Saina</t>
         </is>
       </c>
-      <c r="E55" s="19" t="inlineStr">
-        <is>
-          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
+      <c r="E55" s="16" t="inlineStr">
+        <is>
+          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Indian young woman about 20, sports wear, racket. Full body, standing, facing camera. Plain bright green (#00FF00) background, no text, no shadow.</t>
         </is>
       </c>
     </row>
@@ -63605,29 +63605,29 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="16" t="inlineStr">
-        <is>
-          <t>A024_V_PANDEY</t>
-        </is>
-      </c>
-      <c r="B57" s="16" t="inlineStr">
+      <c r="A57" s="19" t="inlineStr">
+        <is>
+          <t>C04-008_GUPTA_SLUMPED</t>
+        </is>
+      </c>
+      <c r="B57" s="19" t="inlineStr">
         <is>
           <t>A024</t>
         </is>
       </c>
-      <c r="C57" s="16" t="inlineStr">
+      <c r="C57" s="19" t="inlineStr">
         <is>
           <t>Victim</t>
         </is>
       </c>
-      <c r="D57" s="16" t="inlineStr">
+      <c r="D57" s="19" t="inlineStr">
         <is>
           <t>Indian science teacher Ramesh Pandey, about 55, sweater, spectacles, slumped on a study chair, eyes closed</t>
         </is>
       </c>
-      <c r="E57" s="16" t="inlineStr">
-        <is>
-          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Indian science teacher Ramesh Pandey, about 55, sweater, spectacles, slumped on a study chair, eyes closed. Peaceful pose, YouTube-safe: no blood, no wounds. Plain bright green (#00FF00) background, no text, no shadow.</t>
+      <c r="E57" s="19" t="inlineStr">
+        <is>
+          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
         </is>
       </c>
     </row>
@@ -63769,7 +63769,7 @@
     <row r="63">
       <c r="A63" s="19" t="inlineStr">
         <is>
-          <t>C010_SUNITA</t>
+          <t>G_W_MAROON_SAREE_CUT</t>
         </is>
       </c>
       <c r="B63" s="19" t="inlineStr">
@@ -63823,7 +63823,7 @@
     <row r="65">
       <c r="A65" s="19" t="inlineStr">
         <is>
-          <t>C004_BEHEN</t>
+          <t>C002_RIYA_CUT</t>
         </is>
       </c>
       <c r="B65" s="19" t="inlineStr">
@@ -63850,7 +63850,7 @@
     <row r="66">
       <c r="A66" s="19" t="inlineStr">
         <is>
-          <t>C004_PADOSI</t>
+          <t>C12-010_MAHESH</t>
         </is>
       </c>
       <c r="B66" s="19" t="inlineStr">
@@ -63877,7 +63877,7 @@
     <row r="67">
       <c r="A67" s="19" t="inlineStr">
         <is>
-          <t>G_V_MAN_BLUE_CUT</t>
+          <t>C003_SURAJ_CUT</t>
         </is>
       </c>
       <c r="B67" s="19" t="inlineStr">
@@ -63904,7 +63904,7 @@
     <row r="68">
       <c r="A68" s="19" t="inlineStr">
         <is>
-          <t>G_M_YELLOW_KURTA_CUT</t>
+          <t>C001_ROHIT</t>
         </is>
       </c>
       <c r="B68" s="19" t="inlineStr">
@@ -63958,7 +63958,7 @@
     <row r="70">
       <c r="A70" s="19" t="inlineStr">
         <is>
-          <t>G_M_LIGHTMAN_CUT</t>
+          <t>G_M_BLUE_SHIRT_CUT</t>
         </is>
       </c>
       <c r="B70" s="19" t="inlineStr">
@@ -64010,29 +64010,29 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="16" t="inlineStr">
-        <is>
-          <t>A025_V_KHAN</t>
-        </is>
-      </c>
-      <c r="B72" s="16" t="inlineStr">
+      <c r="A72" s="19" t="inlineStr">
+        <is>
+          <t>G_V_MAN_CHECK_CUT</t>
+        </is>
+      </c>
+      <c r="B72" s="19" t="inlineStr">
         <is>
           <t>A025</t>
         </is>
       </c>
-      <c r="C72" s="16" t="inlineStr">
+      <c r="C72" s="19" t="inlineStr">
         <is>
           <t>Victim</t>
         </is>
       </c>
-      <c r="D72" s="16" t="inlineStr">
+      <c r="D72" s="19" t="inlineStr">
         <is>
           <t>Indian wildlife photographer Imtiaz Khan, about 55, khaki shirt, slumped on a sofa near camera gear, eyes closed</t>
         </is>
       </c>
-      <c r="E72" s="16" t="inlineStr">
-        <is>
-          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Indian wildlife photographer Imtiaz Khan, about 55, khaki shirt, slumped on a sofa near camera gear, eyes closed. Peaceful pose, YouTube-safe: no blood, no wounds. Plain bright green (#00FF00) background, no text, no shadow.</t>
+      <c r="E72" s="19" t="inlineStr">
+        <is>
+          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
         </is>
       </c>
     </row>
@@ -64174,7 +64174,7 @@
     <row r="78">
       <c r="A78" s="19" t="inlineStr">
         <is>
-          <t>C001_ROHIT</t>
+          <t>G_CR_ROHIT_CUT</t>
         </is>
       </c>
       <c r="B78" s="19" t="inlineStr">
@@ -64201,7 +64201,7 @@
     <row r="79">
       <c r="A79" s="19" t="inlineStr">
         <is>
-          <t>G_M_BROWN_JACKET_CUT</t>
+          <t>G_M_CAMERA_CUT</t>
         </is>
       </c>
       <c r="B79" s="19" t="inlineStr">
@@ -64228,7 +64228,7 @@
     <row r="80">
       <c r="A80" s="19" t="inlineStr">
         <is>
-          <t>C004_SNEHA</t>
+          <t>C002_POOJA</t>
         </is>
       </c>
       <c r="B80" s="19" t="inlineStr">
@@ -64253,36 +64253,36 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="16" t="inlineStr">
-        <is>
-          <t>A025_BHUPENDRA</t>
-        </is>
-      </c>
-      <c r="B81" s="16" t="inlineStr">
+      <c r="A81" s="19" t="inlineStr">
+        <is>
+          <t>G_KALLU_CUT</t>
+        </is>
+      </c>
+      <c r="B81" s="19" t="inlineStr">
         <is>
           <t>A025</t>
         </is>
       </c>
-      <c r="C81" s="16" t="inlineStr">
+      <c r="C81" s="19" t="inlineStr">
         <is>
           <t>Suspect</t>
         </is>
       </c>
-      <c r="D81" s="16" t="inlineStr">
-        <is>
-          <t>Guide Bhupendra</t>
-        </is>
-      </c>
-      <c r="E81" s="16" t="inlineStr">
-        <is>
-          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Rajasthani guide about 40, safari uniform, turban. Full body, standing, facing camera. Plain bright green (#00FF00) background, no text, no shadow.</t>
+      <c r="D81" s="19" t="inlineStr">
+        <is>
+          <t>Guide Kallu</t>
+        </is>
+      </c>
+      <c r="E81" s="19" t="inlineStr">
+        <is>
+          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="19" t="inlineStr">
         <is>
-          <t>C001_ANJALI</t>
+          <t>C011_EMMA</t>
         </is>
       </c>
       <c r="B82" s="19" t="inlineStr">
@@ -64309,7 +64309,7 @@
     <row r="83">
       <c r="A83" s="19" t="inlineStr">
         <is>
-          <t>G_V_MAN_SHERWANI_CUT</t>
+          <t>C013_LAWYER</t>
         </is>
       </c>
       <c r="B83" s="19" t="inlineStr">
@@ -64442,29 +64442,29 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="16" t="inlineStr">
-        <is>
-          <t>A026_V_TSERING</t>
-        </is>
-      </c>
-      <c r="B88" s="16" t="inlineStr">
+      <c r="A88" s="19" t="inlineStr">
+        <is>
+          <t>C001_VIKAS</t>
+        </is>
+      </c>
+      <c r="B88" s="19" t="inlineStr">
         <is>
           <t>A026</t>
         </is>
       </c>
-      <c r="C88" s="16" t="inlineStr">
+      <c r="C88" s="19" t="inlineStr">
         <is>
           <t>Victim</t>
         </is>
       </c>
-      <c r="D88" s="16" t="inlineStr">
+      <c r="D88" s="19" t="inlineStr">
         <is>
           <t>Sikkimese homestay owner Tsering Bhutia, about 55, traditional bakhu dress, slumped near a fireplace, eyes closed</t>
         </is>
       </c>
-      <c r="E88" s="16" t="inlineStr">
-        <is>
-          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Sikkimese homestay owner Tsering Bhutia, about 55, traditional bakhu dress, slumped near a fireplace, eyes closed. Peaceful pose, YouTube-safe: no blood, no wounds. Plain bright green (#00FF00) background, no text, no shadow.</t>
+      <c r="E88" s="19" t="inlineStr">
+        <is>
+          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
         </is>
       </c>
     </row>
@@ -64577,29 +64577,29 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="18" t="inlineStr">
-        <is>
-          <t>P_A026_SHOES</t>
-        </is>
-      </c>
-      <c r="B93" s="18" t="inlineStr">
+      <c r="A93" s="19" t="inlineStr">
+        <is>
+          <t>P_SHOES</t>
+        </is>
+      </c>
+      <c r="B93" s="19" t="inlineStr">
         <is>
           <t>A026</t>
         </is>
       </c>
-      <c r="C93" s="18" t="inlineStr">
+      <c r="C93" s="19" t="inlineStr">
         <is>
           <t>Saboot (prop)</t>
         </is>
       </c>
-      <c r="D93" s="18" t="inlineStr">
+      <c r="D93" s="19" t="inlineStr">
         <is>
           <t>Snowy trekking shoes near the door</t>
         </is>
       </c>
-      <c r="E93" s="18" t="inlineStr">
-        <is>
-          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Snowy trekking shoes near the door. Close-up object, centered. Plain bright green (#00FF00) background, no text, no shadow.</t>
+      <c r="E93" s="19" t="inlineStr">
+        <is>
+          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
         </is>
       </c>
     </row>
@@ -64633,7 +64633,7 @@
     <row r="95">
       <c r="A95" s="19" t="inlineStr">
         <is>
-          <t>C008_NEHA</t>
+          <t>G_TANVI</t>
         </is>
       </c>
       <c r="B95" s="19" t="inlineStr">
@@ -64648,7 +64648,7 @@
       </c>
       <c r="D95" s="19" t="inlineStr">
         <is>
-          <t>Blogger Neha</t>
+          <t>Blogger Tanvi</t>
         </is>
       </c>
       <c r="E95" s="19" t="inlineStr">
@@ -64660,7 +64660,7 @@
     <row r="96">
       <c r="A96" s="19" t="inlineStr">
         <is>
-          <t>G_M_CAMERA_CUT</t>
+          <t>G_M_BROWN_JACKET_CUT</t>
         </is>
       </c>
       <c r="B96" s="19" t="inlineStr">
@@ -64685,36 +64685,36 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="16" t="inlineStr">
-        <is>
-          <t>A026_KARMA</t>
-        </is>
-      </c>
-      <c r="B97" s="16" t="inlineStr">
+      <c r="A97" s="19" t="inlineStr">
+        <is>
+          <t>G_M_BLUE_JACKET_B_CUT</t>
+        </is>
+      </c>
+      <c r="B97" s="19" t="inlineStr">
         <is>
           <t>A026</t>
         </is>
       </c>
-      <c r="C97" s="16" t="inlineStr">
+      <c r="C97" s="19" t="inlineStr">
         <is>
           <t>Suspect</t>
         </is>
       </c>
-      <c r="D97" s="16" t="inlineStr">
+      <c r="D97" s="19" t="inlineStr">
         <is>
           <t>Beta Karma (homestay bechne par jhagda)</t>
         </is>
       </c>
-      <c r="E97" s="16" t="inlineStr">
-        <is>
-          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Sikkimese young man about 27, jacket. Full body, standing, facing camera. Plain bright green (#00FF00) background, no text, no shadow.</t>
+      <c r="E97" s="19" t="inlineStr">
+        <is>
+          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="19" t="inlineStr">
         <is>
-          <t>G_M_OLD_GLASSES_CUT</t>
+          <t>C006_GUPTA</t>
         </is>
       </c>
       <c r="B98" s="19" t="inlineStr">
@@ -64741,7 +64741,7 @@
     <row r="99">
       <c r="A99" s="19" t="inlineStr">
         <is>
-          <t>C002_RIYA_CUT</t>
+          <t>C001_ANJALI</t>
         </is>
       </c>
       <c r="B99" s="19" t="inlineStr">
@@ -64768,7 +64768,7 @@
     <row r="100">
       <c r="A100" s="19" t="inlineStr">
         <is>
-          <t>C16-001_DRMEHTA</t>
+          <t>G_M_OLD_GLASSES_CUT</t>
         </is>
       </c>
       <c r="B100" s="19" t="inlineStr">
@@ -64793,36 +64793,36 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="16" t="inlineStr">
-        <is>
-          <t>A026_DORJEE</t>
-        </is>
-      </c>
-      <c r="B101" s="16" t="inlineStr">
+      <c r="A101" s="19" t="inlineStr">
+        <is>
+          <t>G_M_APRON_CUT</t>
+        </is>
+      </c>
+      <c r="B101" s="19" t="inlineStr">
         <is>
           <t>A026</t>
         </is>
       </c>
-      <c r="C101" s="16" t="inlineStr">
+      <c r="C101" s="19" t="inlineStr">
         <is>
           <t>Suspect</t>
         </is>
       </c>
-      <c r="D101" s="16" t="inlineStr">
+      <c r="D101" s="19" t="inlineStr">
         <is>
           <t>Cook Dorjee (daan peti ki chaabi)</t>
         </is>
       </c>
-      <c r="E101" s="16" t="inlineStr">
-        <is>
-          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Sikkimese cook about 45, apron. Full body, standing, facing camera. Plain bright green (#00FF00) background, no text, no shadow.</t>
+      <c r="E101" s="19" t="inlineStr">
+        <is>
+          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="19" t="inlineStr">
         <is>
-          <t>C007_VIKRAM</t>
+          <t>G_CIVIL_BLACK_CUT</t>
         </is>
       </c>
       <c r="B102" s="19" t="inlineStr">
@@ -64874,29 +64874,29 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="16" t="inlineStr">
-        <is>
-          <t>A027_V_MOHAPATRA</t>
-        </is>
-      </c>
-      <c r="B104" s="16" t="inlineStr">
+      <c r="A104" s="19" t="inlineStr">
+        <is>
+          <t>G_V_MAN_SHERWANI_CUT</t>
+        </is>
+      </c>
+      <c r="B104" s="19" t="inlineStr">
         <is>
           <t>A027</t>
         </is>
       </c>
-      <c r="C104" s="16" t="inlineStr">
+      <c r="C104" s="19" t="inlineStr">
         <is>
           <t>Victim</t>
         </is>
       </c>
-      <c r="D104" s="16" t="inlineStr">
+      <c r="D104" s="19" t="inlineStr">
         <is>
           <t>Indian museum curator Dr. Bijay Mohapatra, about 60, kurta and spectacles, slumped near a glass display case, eyes closed</t>
         </is>
       </c>
-      <c r="E104" s="16" t="inlineStr">
-        <is>
-          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Indian museum curator Dr. Bijay Mohapatra, about 60, kurta and spectacles, slumped near a glass display case, eyes closed. Peaceful pose, YouTube-safe: no blood, no wounds. Plain bright green (#00FF00) background, no text, no shadow.</t>
+      <c r="E104" s="19" t="inlineStr">
+        <is>
+          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
         </is>
       </c>
     </row>
@@ -65038,7 +65038,7 @@
     <row r="110">
       <c r="A110" s="19" t="inlineStr">
         <is>
-          <t>C002_POOJA</t>
+          <t>C019_COWORKER</t>
         </is>
       </c>
       <c r="B110" s="19" t="inlineStr">
@@ -65092,7 +65092,7 @@
     <row r="112">
       <c r="A112" s="19" t="inlineStr">
         <is>
-          <t>C18-003_PRATEEK</t>
+          <t>C10-004_DEEPAK</t>
         </is>
       </c>
       <c r="B112" s="19" t="inlineStr">
@@ -65119,7 +65119,7 @@
     <row r="113">
       <c r="A113" s="19" t="inlineStr">
         <is>
-          <t>C17-001_SETH</t>
+          <t>C017_BESTMAN</t>
         </is>
       </c>
       <c r="B113" s="19" t="inlineStr">
@@ -65146,7 +65146,7 @@
     <row r="114">
       <c r="A114" s="19" t="inlineStr">
         <is>
-          <t>G_V_WOMAN_SAREE_CUT</t>
+          <t>C010_SUNITA</t>
         </is>
       </c>
       <c r="B114" s="19" t="inlineStr">
@@ -65173,7 +65173,7 @@
     <row r="115">
       <c r="A115" s="19" t="inlineStr">
         <is>
-          <t>G_V_MAN_CHECK_CUT</t>
+          <t>C005_VICKY</t>
         </is>
       </c>
       <c r="B115" s="19" t="inlineStr">
@@ -65200,7 +65200,7 @@
     <row r="116">
       <c r="A116" s="19" t="inlineStr">
         <is>
-          <t>C007_KAVYA</t>
+          <t>C004_BEHEN</t>
         </is>
       </c>
       <c r="B116" s="19" t="inlineStr">
@@ -65227,7 +65227,7 @@
     <row r="117">
       <c r="A117" s="19" t="inlineStr">
         <is>
-          <t>G_V_MAN_GREY_CUT</t>
+          <t>C007_NIKHIL</t>
         </is>
       </c>
       <c r="B117" s="19" t="inlineStr">
@@ -65281,7 +65281,7 @@
     <row r="119">
       <c r="A119" s="19" t="inlineStr">
         <is>
-          <t>G_RAMU</t>
+          <t>G_M_GAMCHHA_CUT</t>
         </is>
       </c>
       <c r="B119" s="19" t="inlineStr">
@@ -65296,7 +65296,7 @@
       </c>
       <c r="D119" s="19" t="inlineStr">
         <is>
-          <t>Safaiwala Ramu</t>
+          <t>Safaiwala Gopi</t>
         </is>
       </c>
       <c r="E119" s="19" t="inlineStr">
@@ -65333,29 +65333,29 @@
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="16" t="inlineStr">
-        <is>
-          <t>A028_V_GREWAL</t>
-        </is>
-      </c>
-      <c r="B121" s="16" t="inlineStr">
+      <c r="A121" s="19" t="inlineStr">
+        <is>
+          <t>C08-007_KAPOOR</t>
+        </is>
+      </c>
+      <c r="B121" s="19" t="inlineStr">
         <is>
           <t>A028</t>
         </is>
       </c>
-      <c r="C121" s="16" t="inlineStr">
+      <c r="C121" s="19" t="inlineStr">
         <is>
           <t>Victim</t>
         </is>
       </c>
-      <c r="D121" s="16" t="inlineStr">
+      <c r="D121" s="19" t="inlineStr">
         <is>
           <t>Indian hospital owner Dr. Harjeet Grewal, about 60, white coat, slumped on his cabin chair, eyes closed</t>
         </is>
       </c>
-      <c r="E121" s="16" t="inlineStr">
-        <is>
-          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Indian hospital owner Dr. Harjeet Grewal, about 60, white coat, slumped on his cabin chair, eyes closed. Peaceful pose, YouTube-safe: no blood, no wounds. Plain bright green (#00FF00) background, no text, no shadow.</t>
+      <c r="E121" s="19" t="inlineStr">
+        <is>
+          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
         </is>
       </c>
     </row>
@@ -65497,7 +65497,7 @@
     <row r="127">
       <c r="A127" s="19" t="inlineStr">
         <is>
-          <t>C005_VICKY</t>
+          <t>C018_BOYFRIEND</t>
         </is>
       </c>
       <c r="B127" s="19" t="inlineStr">
@@ -65684,29 +65684,29 @@
       </c>
     </row>
     <row r="134">
-      <c r="A134" s="19" t="inlineStr">
-        <is>
-          <t>C001_ANJALI</t>
-        </is>
-      </c>
-      <c r="B134" s="19" t="inlineStr">
+      <c r="A134" s="16" t="inlineStr">
+        <is>
+          <t>A028_ANU</t>
+        </is>
+      </c>
+      <c r="B134" s="16" t="inlineStr">
         <is>
           <t>A028</t>
         </is>
       </c>
-      <c r="C134" s="19" t="inlineStr">
+      <c r="C134" s="16" t="inlineStr">
         <is>
           <t>Suspect</t>
         </is>
       </c>
-      <c r="D134" s="19" t="inlineStr">
+      <c r="D134" s="16" t="inlineStr">
         <is>
           <t>Yoga teacher Anu</t>
         </is>
       </c>
-      <c r="E134" s="19" t="inlineStr">
-        <is>
-          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
+      <c r="E134" s="16" t="inlineStr">
+        <is>
+          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Indian woman about 35, yoga wear. Full body, standing, facing camera. Plain bright green (#00FF00) background, no text, no shadow.</t>
         </is>
       </c>
     </row>
@@ -65740,7 +65740,7 @@
     <row r="136">
       <c r="A136" s="19" t="inlineStr">
         <is>
-          <t>C04-008_GUPTA_SLUMPED</t>
+          <t>C17-001_SETH</t>
         </is>
       </c>
       <c r="B136" s="19" t="inlineStr">
@@ -65902,7 +65902,7 @@
     <row r="142">
       <c r="A142" s="19" t="inlineStr">
         <is>
-          <t>C006_GUPTA</t>
+          <t>G_M_OLD_NOGLASSES_CUT</t>
         </is>
       </c>
       <c r="B142" s="19" t="inlineStr">
@@ -65929,7 +65929,7 @@
     <row r="143">
       <c r="A143" s="19" t="inlineStr">
         <is>
-          <t>C004_AMIT</t>
+          <t>C003_BHATIJA</t>
         </is>
       </c>
       <c r="B143" s="19" t="inlineStr">
@@ -65956,7 +65956,7 @@
     <row r="144">
       <c r="A144" s="19" t="inlineStr">
         <is>
-          <t>C004_SNEHA</t>
+          <t>C002_POOJA</t>
         </is>
       </c>
       <c r="B144" s="19" t="inlineStr">
@@ -65983,7 +65983,7 @@
     <row r="145">
       <c r="A145" s="19" t="inlineStr">
         <is>
-          <t>C003_BHATIJA</t>
+          <t>C004_AMIT</t>
         </is>
       </c>
       <c r="B145" s="19" t="inlineStr">
@@ -66010,7 +66010,7 @@
     <row r="146">
       <c r="A146" s="19" t="inlineStr">
         <is>
-          <t>G_V_MAN_BLUE_CUT</t>
+          <t>G_M_BLUE_JACKET_A_CUT</t>
         </is>
       </c>
       <c r="B146" s="19" t="inlineStr">
@@ -66064,7 +66064,7 @@
     <row r="148">
       <c r="A148" s="19" t="inlineStr">
         <is>
-          <t>C08-004_MR_RATHI</t>
+          <t>C004_PADOSI</t>
         </is>
       </c>
       <c r="B148" s="19" t="inlineStr">
@@ -66170,29 +66170,29 @@
       </c>
     </row>
     <row r="152">
-      <c r="A152" s="16" t="inlineStr">
-        <is>
-          <t>A030_V_JOSHI</t>
-        </is>
-      </c>
-      <c r="B152" s="16" t="inlineStr">
+      <c r="A152" s="19" t="inlineStr">
+        <is>
+          <t>C04-010_ARJUN</t>
+        </is>
+      </c>
+      <c r="B152" s="19" t="inlineStr">
         <is>
           <t>A030</t>
         </is>
       </c>
-      <c r="C152" s="16" t="inlineStr">
+      <c r="C152" s="19" t="inlineStr">
         <is>
           <t>Victim</t>
         </is>
       </c>
-      <c r="D152" s="16" t="inlineStr">
+      <c r="D152" s="19" t="inlineStr">
         <is>
           <t>Indian astronomer Dr. Prakash Joshi, about 62, woollen sweater, slumped near a telescope, eyes closed</t>
         </is>
       </c>
-      <c r="E152" s="16" t="inlineStr">
-        <is>
-          <t>Flat 2D cartoon illustration, bold black outlines, same art style as the 'Detective Shivam' series, Indian setting, warm cinematic colours, no watermark. Indian astronomer Dr. Prakash Joshi, about 62, woollen sweater, slumped near a telescope, eyes closed. Peaceful pose, YouTube-safe: no blood, no wounds. Plain bright green (#00FF00) background, no text, no shadow.</t>
+      <c r="E152" s="19" t="inlineStr">
+        <is>
+          <t>PEHLE SE HAI (purani image, nayi mat banao) – ek baar dekh lo look role se mel khaata hai</t>
         </is>
       </c>
     </row>
@@ -66334,7 +66334,7 @@
     <row r="158">
       <c r="A158" s="19" t="inlineStr">
         <is>
-          <t>G_M_GREY_HOODIE_CUT</t>
+          <t>C020_BROTHER</t>
         </is>
       </c>
       <c r="B158" s="19" t="inlineStr">
@@ -66361,7 +66361,7 @@
     <row r="159">
       <c r="A159" s="19" t="inlineStr">
         <is>
-          <t>C005_NEHA</t>
+          <t>G_W_PINK_SUIT_CUT</t>
         </is>
       </c>
       <c r="B159" s="19" t="inlineStr">
@@ -66388,7 +66388,7 @@
     <row r="160">
       <c r="A160" s="19" t="inlineStr">
         <is>
-          <t>G_M_OLD_NOGLASSES_CUT</t>
+          <t>C011_TOM</t>
         </is>
       </c>
       <c r="B160" s="19" t="inlineStr">
@@ -66415,7 +66415,7 @@
     <row r="161">
       <c r="A161" s="19" t="inlineStr">
         <is>
-          <t>C007_KAVYA</t>
+          <t>C018_SISTER</t>
         </is>
       </c>
       <c r="B161" s="19" t="inlineStr">
@@ -66523,7 +66523,7 @@
     <row r="165">
       <c r="A165" s="19" t="inlineStr">
         <is>
-          <t>C10-004_DEEPAK</t>
+          <t>C03-003_VICKY</t>
         </is>
       </c>
       <c r="B165" s="19" t="inlineStr">
@@ -66577,7 +66577,7 @@
     <row r="167">
       <c r="A167" s="19" t="inlineStr">
         <is>
-          <t>G_V_MAN_CHECK_CUT</t>
+          <t>C008_GUEST</t>
         </is>
       </c>
       <c r="B167" s="19" t="inlineStr">

</xml_diff>